<commit_message>
Replace BOQ Image1 with reprofilage sector items
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/Bordereau_prix_drainage_par_secteur.xlsx
+++ b/engineering/stormwater-pumping/Bordereau_prix_drainage_par_secteur.xlsx
@@ -91,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -109,6 +109,15 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -474,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -642,17 +651,17 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>DEM-001</t>
+          <t>SCI-001</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Decoupage et demolition de pavage / asphalte</t>
+          <t>Sciage de pavage</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D8" s="4">
@@ -666,7 +675,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Secteurs A / raccordements</t>
+          <t>Zone de reprofilage</t>
         </is>
       </c>
       <c r="H8" s="5" t="n"/>
@@ -674,17 +683,17 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>EXC-001</t>
+          <t>DEM-001</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Excavation de tranchee pour reseau pluvial</t>
+          <t>Enlevement de pavage</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="D9" s="4">
@@ -698,7 +707,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Tous secteurs</t>
+          <t>Zone de reprofilage / secteurs A</t>
         </is>
       </c>
       <c r="H9" s="5" t="n"/>
@@ -706,17 +715,17 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>EXC-002</t>
+          <t>EXC-001</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Hydro-excavation pour localisation de conduites existantes</t>
+          <t>Excavation de tranchee pour reseau pluvial</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>h</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="D10" s="4">
@@ -730,7 +739,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Secteur P-01 / P-02 / raccord Ø1800</t>
+          <t>Tous secteurs</t>
         </is>
       </c>
       <c r="H10" s="5" t="n"/>
@@ -738,17 +747,17 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>CAN-300</t>
+          <t>EXC-002</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Fourniture et pose conduite pluviale DN300</t>
+          <t>Hydro-excavation pour localisation de conduites existantes</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>h</t>
         </is>
       </c>
       <c r="D11" s="4">
@@ -762,7 +771,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Schema hydraulique principal</t>
+          <t>Secteur P-01 / P-02 / raccord Ø1800</t>
         </is>
       </c>
       <c r="H11" s="5" t="n"/>
@@ -770,12 +779,12 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>CAN-375</t>
+          <t>CAN-300</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Fourniture et pose raccord / conduite DN375</t>
+          <t>Fourniture et pose conduite pluviale DN300</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -794,7 +803,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Raccord propose</t>
+          <t>Secteurs avec conduites nouvelles</t>
         </is>
       </c>
       <c r="H12" s="5" t="n"/>
@@ -802,17 +811,17 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>REG-001</t>
+          <t>CAN-375</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Regard RP-01 (ajustement / reconstruction locale)</t>
+          <t>Fourniture et pose raccord / conduite DN375</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D13" s="4">
@@ -826,7 +835,7 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Noeud de repartition</t>
+          <t>Raccord propose</t>
         </is>
       </c>
       <c r="H13" s="5" t="n"/>
@@ -834,12 +843,12 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>REG-002</t>
+          <t>REG-001</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Regard RP-02 avec clapet anti-retour</t>
+          <t>Regard RP-01 (ajustement / reconstruction locale)</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -858,7 +867,7 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Aval poste de pompage</t>
+          <t>Noeud de repartition</t>
         </is>
       </c>
       <c r="H14" s="5" t="n"/>
@@ -866,12 +875,12 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>SEP-001</t>
+          <t>REG-002</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Unite de traitement type Jellyfish (DP-01)</t>
+          <t>Regard RP-02 avec clapet anti-retour</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -890,7 +899,7 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Branche traitement</t>
+          <t>Aval poste / reseau existant</t>
         </is>
       </c>
       <c r="H15" s="5" t="n"/>
@@ -898,12 +907,12 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>PUI-001</t>
+          <t>SEP-001</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Nouveau puisard</t>
+          <t>Unite de traitement type Jellyfish (DP-01)</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -922,7 +931,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Secteur A</t>
+          <t>Branche traitement</t>
         </is>
       </c>
       <c r="H16" s="5" t="n"/>
@@ -930,17 +939,17 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>BOR-001</t>
+          <t>PUI-001</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Saignee dans bordure / raccord de bordure</t>
+          <t>Nouveau puisard</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>u</t>
         </is>
       </c>
       <c r="D17" s="4">
@@ -962,17 +971,17 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>RAC-001</t>
+          <t>BOR-001</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Raccordement a la conduite existante Ø1800</t>
+          <t>Saignee dans bordure / raccord de bordure</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D18" s="4">
@@ -986,7 +995,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Secteur P-01 / P-02</t>
+          <t>Secteur A</t>
         </is>
       </c>
       <c r="H18" s="5" t="n"/>
@@ -994,17 +1003,17 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>REM-001</t>
+          <t>BORD-001</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Remblai compacte et remise en forme</t>
+          <t>Reconstruction de bordure (si requise)</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D19" s="4">
@@ -1018,7 +1027,7 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Tous secteurs</t>
+          <t>Zone de reprofilage</t>
         </is>
       </c>
       <c r="H19" s="5" t="n"/>
@@ -1026,17 +1035,17 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>PAV-001</t>
+          <t>RAC-001</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Reprofilage / reprise de pavage</t>
+          <t>Raccordement a la conduite existante Ø1800</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>u</t>
         </is>
       </c>
       <c r="D20" s="4">
@@ -1050,7 +1059,7 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Secteurs a risque drainage</t>
+          <t>Secteur P-01 / P-02</t>
         </is>
       </c>
       <c r="H20" s="5" t="n"/>
@@ -1058,17 +1067,17 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>ESS-001</t>
+          <t>REM-001</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Essais / verification hydraulique et mise en service</t>
+          <t>Remblai et materiaux granulaires</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="D21" s="4">
@@ -1082,7 +1091,7 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Reseau pluvial</t>
+          <t>Tous secteurs</t>
         </is>
       </c>
       <c r="H21" s="5" t="n"/>
@@ -1090,17 +1099,17 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>DOC-001</t>
+          <t>PAV-001</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Plans finaux / dossier de recollement</t>
+          <t>Reprofilage / reprise de pavage</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="D22" s="4">
@@ -1114,19 +1123,147 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
+          <t>Secteurs a risque drainage</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>REF-001</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Refection des surfaces (gazon, etc.)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="D23" s="4">
+        <f>SUMIFS(Detail_Image1!$H:$H,Detail_Image1!$C:$C,$A23)+SUMIFS(Detail_Image2!$H:$H,Detail_Image2!$C:$C,$A23)+SUMIFS(Detail_Image3!$H:$H,Detail_Image3!$C:$C,$A23)+SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A23)</f>
+        <v/>
+      </c>
+      <c r="E23" s="4" t="n"/>
+      <c r="F23" s="4">
+        <f>IF(E23="","",D23*E23)</f>
+        <v/>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>Zone de reprofilage / finitions</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>AJU-001</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Ajustement d'ouvrages existants</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+      <c r="D24" s="9">
+        <f>SUMIFS(Detail_Image1!$H:$H,Detail_Image1!$C:$C,$A24)+SUMIFS(Detail_Image2!$H:$H,Detail_Image2!$C:$C,$A24)+SUMIFS(Detail_Image3!$H:$H,Detail_Image3!$C:$C,$A24)+SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A24)</f>
+        <v/>
+      </c>
+      <c r="E24" s="4" t="n"/>
+      <c r="F24" s="9">
+        <f>IF(E24="","",D24*E24)</f>
+        <v/>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Zone de reprofilage / reseau existant</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>ESS-001</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Essais / verification hydraulique et mise en service</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="D25" s="4">
+        <f>SUMIFS(Detail_Image1!$H:$H,Detail_Image1!$C:$C,$A25)+SUMIFS(Detail_Image2!$H:$H,Detail_Image2!$C:$C,$A25)+SUMIFS(Detail_Image3!$H:$H,Detail_Image3!$C:$C,$A25)+SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A25)</f>
+        <v/>
+      </c>
+      <c r="E25" s="4" t="n"/>
+      <c r="F25" s="4">
+        <f>IF(E25="","",D25*E25)</f>
+        <v/>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Reseau pluvial</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>DOC-001</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Plans finaux / dossier de recollement</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="D26" s="4">
+        <f>SUMIFS(Detail_Image1!$H:$H,Detail_Image1!$C:$C,$A26)+SUMIFS(Detail_Image2!$H:$H,Detail_Image2!$C:$C,$A26)+SUMIFS(Detail_Image3!$H:$H,Detail_Image3!$C:$C,$A26)+SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A26)</f>
+        <v/>
+      </c>
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4">
+        <f>IF(E26="","",D26*E26)</f>
+        <v/>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
           <t>Tous secteurs</t>
         </is>
       </c>
-      <c r="H22" s="5" t="n"/>
-    </row>
-    <row r="24">
-      <c r="D24" s="6" t="inlineStr">
+      <c r="H26" s="5" t="n"/>
+    </row>
+    <row r="28">
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="F24" s="6">
-        <f>SUM(F5:F22)</f>
+      <c r="F28" s="9">
+        <f>SUM(F5:F26)</f>
         <v/>
       </c>
     </row>
@@ -1163,7 +1300,7 @@
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>Detail quantites - Detail_Image1</t>
+          <t>Detail quantites - Image1 (zone de reprofilage)</t>
         </is>
       </c>
     </row>
@@ -1222,22 +1359,22 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Image1</t>
+          <t>Image1_reprofilage</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Troncon S1</t>
+          <t>Zone de reprofilage</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>CAN-300</t>
+          <t>SCI-001</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Conduite DN300 StormBrixx -&gt; RP-01</t>
+          <t>Sciage de pavage</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -1246,7 +1383,7 @@
         </is>
       </c>
       <c r="F4" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G4" s="4" t="n">
         <v>1</v>
@@ -1257,7 +1394,7 @@
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Mesure lue sur schema hydraulique</t>
+          <t>Longueur a mesurer sur plan DAO/PDF</t>
         </is>
       </c>
       <c r="J4" s="5" t="n"/>
@@ -1265,31 +1402,31 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Image1</t>
+          <t>Image1_reprofilage</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Troncon S2</t>
+          <t>Zone de reprofilage</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>CAN-300</t>
+          <t>DEM-001</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Conduite DN300 RP-01 -&gt; point de convergence</t>
+          <t>Enlevement de pavage</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G5" s="4" t="n">
         <v>1</v>
@@ -1300,7 +1437,7 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Mesure lue sur schema hydraulique</t>
+          <t>Surface a confirmer par metrage</t>
         </is>
       </c>
       <c r="J5" s="5" t="n"/>
@@ -1308,22 +1445,22 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Image1</t>
+          <t>Image1_reprofilage</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Troncon S3</t>
+          <t>Zone de reprofilage</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>CAN-300</t>
+          <t>BORD-001</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Conduite DN300 vers DP-01 (branche derivee)</t>
+          <t>Reconstruction de bordure (si requise)</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -1332,7 +1469,7 @@
         </is>
       </c>
       <c r="F6" s="4" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="G6" s="4" t="n">
         <v>1</v>
@@ -1343,7 +1480,7 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Mesure lue sur schema hydraulique</t>
+          <t>Longueur conditionnelle selon etat existant</t>
         </is>
       </c>
       <c r="J6" s="5" t="n"/>
@@ -1351,31 +1488,31 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Image1</t>
+          <t>Image1_reprofilage</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Troncon S4</t>
+          <t>Zone de reprofilage</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>CAN-300</t>
+          <t>REM-001</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Conduite DN300 retour DP-01 -&gt; convergence</t>
+          <t>Remblai et materiaux granulaires</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="G7" s="4" t="n">
         <v>1</v>
@@ -1386,7 +1523,7 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Mesure a confirmer sur plan IFC</t>
+          <t>Volume apres profils et epaisseur finale</t>
         </is>
       </c>
       <c r="J7" s="5" t="n"/>
@@ -1394,31 +1531,31 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Image1</t>
+          <t>Image1_reprofilage</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Troncon S5</t>
+          <t>Zone de reprofilage</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>CAN-300</t>
+          <t>AJU-001</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Conduite DN300 convergence -&gt; RP-02</t>
+          <t>Ajustement d'ouvrages existants</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>u</t>
         </is>
       </c>
       <c r="F8" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G8" s="4" t="n">
         <v>1</v>
@@ -1429,7 +1566,7 @@
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Mesure lue sur schema hydraulique</t>
+          <t>Minimum 1 unite, ajuster apres releve terrain</t>
         </is>
       </c>
       <c r="J8" s="5" t="n"/>
@@ -1437,31 +1574,31 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Image1</t>
+          <t>Image1_reprofilage</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Troncon S6</t>
+          <t>Zone de reprofilage</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>CAN-300</t>
+          <t>REF-001</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Conduite DN300 RP-02 -&gt; exutoire gravitaire</t>
+          <t>Refection des surfaces (gazon, etc.)</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>14.5</v>
+        <v>0</v>
       </c>
       <c r="G9" s="4" t="n">
         <v>1</v>
@@ -1472,150 +1609,57 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Mesure lue sur schema hydraulique</t>
+          <t>Surface finale a confirmer</t>
         </is>
       </c>
       <c r="J9" s="5" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Image1</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Noeud RP-01</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>REG-001</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>Regard RP-01 regulateur (ajustement/reprise)</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>u</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="4">
-        <f>IF(F10="","",F10*G10)</f>
-        <v/>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>Quantite minimale = 1</t>
-        </is>
-      </c>
+      <c r="A10" s="4" t="n"/>
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="4" t="n"/>
+      <c r="D10" s="5" t="n"/>
+      <c r="E10" s="4" t="n"/>
+      <c r="F10" s="4" t="n"/>
+      <c r="G10" s="4" t="n"/>
+      <c r="H10" s="4" t="n"/>
+      <c r="I10" s="5" t="n"/>
       <c r="J10" s="5" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Image1</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Branche traitement</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>SEP-001</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Unite de traitement type Jellyfish (DP-01)</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>u</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" s="4">
-        <f>IF(F11="","",F11*G11)</f>
-        <v/>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>Valider modele/fournisseur</t>
-        </is>
-      </c>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Sous-total (controle)</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="4" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="4" t="n"/>
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="11">
+        <f>SUM(H4:H9)</f>
+        <v/>
+      </c>
+      <c r="I11" s="5" t="n"/>
       <c r="J11" s="5" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Image1</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Aval pompage</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>REG-002</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Regard RP-02 avec clapet</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>u</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" s="4">
-        <f>IF(F12="","",F12*G12)</f>
-        <v/>
-      </c>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>Quantite minimale = 1</t>
-        </is>
-      </c>
+      <c r="A12" s="4" t="n"/>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="4" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="4" t="n"/>
+      <c r="F12" s="4" t="n"/>
+      <c r="G12" s="4" t="n"/>
+      <c r="H12" s="4" t="n"/>
+      <c r="I12" s="5" t="n"/>
       <c r="J12" s="5" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>Sous-total (controle)</t>
-        </is>
-      </c>
-      <c r="H14" s="8">
-        <f>SUM(H4:H12)</f>
-        <v/>
-      </c>
+      <c r="A14" s="8" t="n"/>
+      <c r="H14" s="8" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2530,7 +2574,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -2610,6 +2654,13 @@
       <c r="A13" t="inlineStr">
         <is>
           <t>- Remplacer les hypotheses par metrage DAO/terrain des que disponible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>- Detail_Image1 a ete remplace par la zone de reprofilage (items de preparation/refection) selon la nouvelle image.</t>
         </is>
       </c>
     </row>
@@ -2624,7 +2675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2724,100 +2775,100 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>DEM-001</t>
+          <t>SCI-001</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Decoupage et demolition de pavage / asphalte</t>
+          <t>Sciage de pavage</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Secteurs A / raccordements</t>
+          <t>Zone de reprofilage</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>EXC-001</t>
+          <t>DEM-001</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Excavation de tranchee pour reseau pluvial</t>
+          <t>Enlevement de pavage</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Tous secteurs</t>
+          <t>Zone de reprofilage / secteurs A</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>EXC-002</t>
+          <t>EXC-001</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Hydro-excavation pour localisation de conduites existantes</t>
+          <t>Excavation de tranchee pour reseau pluvial</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>h</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Secteur P-01 / P-02 / raccord Ø1800</t>
+          <t>Tous secteurs</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>CAN-300</t>
+          <t>EXC-002</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Fourniture et pose conduite pluviale DN300</t>
+          <t>Hydro-excavation pour localisation de conduites existantes</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>h</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Schema hydraulique principal</t>
+          <t>Secteur P-01 / P-02 / raccord Ø1800</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>CAN-375</t>
+          <t>CAN-300</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Fourniture et pose raccord / conduite DN375</t>
+          <t>Fourniture et pose conduite pluviale DN300</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -2827,41 +2878,41 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Raccord propose</t>
+          <t>Secteurs avec conduites nouvelles</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>REG-001</t>
+          <t>CAN-375</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Regard RP-01 (ajustement / reconstruction locale)</t>
+          <t>Fourniture et pose raccord / conduite DN375</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Noeud de repartition</t>
+          <t>Raccord propose</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>REG-002</t>
+          <t>REG-001</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Regard RP-02 avec clapet anti-retour</t>
+          <t>Regard RP-01 (ajustement / reconstruction locale)</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -2871,19 +2922,19 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Aval poste de pompage</t>
+          <t>Noeud de repartition</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>SEP-001</t>
+          <t>REG-002</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Unite de traitement type Jellyfish (DP-01)</t>
+          <t>Regard RP-02 avec clapet anti-retour</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -2893,19 +2944,19 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Branche traitement</t>
+          <t>Aval poste / reseau existant</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>PUI-001</t>
+          <t>SEP-001</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Nouveau puisard</t>
+          <t>Unite de traitement type Jellyfish (DP-01)</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -2915,24 +2966,24 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Secteur A</t>
+          <t>Branche traitement</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>BOR-001</t>
+          <t>PUI-001</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Saignee dans bordure / raccord de bordure</t>
+          <t>Nouveau puisard</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>u</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -2944,108 +2995,196 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>RAC-001</t>
+          <t>BOR-001</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Raccordement a la conduite existante Ø1800</t>
+          <t>Saignee dans bordure / raccord de bordure</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Secteur P-01 / P-02</t>
+          <t>Secteur A</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>REM-001</t>
+          <t>BORD-001</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Remblai compacte et remise en forme</t>
+          <t>Reconstruction de bordure (si requise)</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Tous secteurs</t>
+          <t>Zone de reprofilage</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>PAV-001</t>
+          <t>RAC-001</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Reprofilage / reprise de pavage</t>
+          <t>Raccordement a la conduite existante Ø1800</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>u</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Secteurs a risque drainage</t>
+          <t>Secteur P-01 / P-02</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>ESS-001</t>
+          <t>REM-001</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Essais / verification hydraulique et mise en service</t>
+          <t>Remblai et materiaux granulaires</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Reseau pluvial</t>
+          <t>Tous secteurs</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
+          <t>PAV-001</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Reprofilage / reprise de pavage</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Secteurs a risque drainage</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>REF-001</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Refection des surfaces (gazon, etc.)</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Zone de reprofilage / finitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>AJU-001</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Ajustement d'ouvrages existants</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Zone de reprofilage / reseau existant</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>ESS-001</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Essais / verification hydraulique et mise en service</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Reseau pluvial</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
           <t>DOC-001</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Plans finaux / dossier de recollement</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>lot</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>Tous secteurs</t>
         </is>

</xml_diff>

<commit_message>
Integrate 557m2 reprofilage image quantities in BOQ
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/Bordereau_prix_drainage_par_secteur.xlsx
+++ b/engineering/stormwater-pumping/Bordereau_prix_drainage_par_secteur.xlsx
@@ -1426,7 +1426,7 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>0</v>
+        <v>557</v>
       </c>
       <c r="G5" s="4" t="n">
         <v>1</v>
@@ -1437,10 +1437,14 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Surface a confirmer par metrage</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="n"/>
+          <t>Image ajoutee: zone delimitee 557 m2</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Hypothese: enlevement sur toute la zone reprise</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -1584,12 +1588,12 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>REF-001</t>
+          <t>PAV-001</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Refection des surfaces (gazon, etc.)</t>
+          <t>Reprofilage / reprise de pavage (point bas a elev. 29,720 m)</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -1598,7 +1602,7 @@
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>0</v>
+        <v>557</v>
       </c>
       <c r="G9" s="4" t="n">
         <v>1</v>
@@ -1609,22 +1613,61 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Surface finale a confirmer</t>
-        </is>
-      </c>
-      <c r="J9" s="5" t="n"/>
+          <t>Image ajoutee: annotation 557 m2 + cote 29,720</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Surface de reprise de pavage selon zone surlignee</t>
+        </is>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="4" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="n"/>
-      <c r="G10" s="4" t="n"/>
-      <c r="H10" s="4" t="n"/>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5" t="n"/>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Image1_reprofilage</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Zone de reprofilage</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>REF-001</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Refection des surfaces (gazon, etc.)</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" s="4">
+        <f>IF(F10="","",F10*G10)</f>
+        <v/>
+      </c>
+      <c r="I10" s="5" t="inlineStr">
+        <is>
+          <t>Si surfaces non pavees sont affectees</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>A ajuster apres verification terrain</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -1639,7 +1682,7 @@
       <c r="F11" s="4" t="n"/>
       <c r="G11" s="4" t="n"/>
       <c r="H11" s="11">
-        <f>SUM(H4:H9)</f>
+        <f>SUM(H4:H10)</f>
         <v/>
       </c>
       <c r="I11" s="5" t="n"/>
@@ -1657,6 +1700,7 @@
       <c r="I12" s="5" t="n"/>
       <c r="J12" s="5" t="n"/>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="8" t="n"/>
       <c r="H14" s="8" t="n"/>

</xml_diff>

<commit_message>
sync BOQ workbook from 42c6582
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/Bordereau_prix_drainage_par_secteur.xlsx
+++ b/engineering/stormwater-pumping/Bordereau_prix_drainage_par_secteur.xlsx
@@ -91,7 +91,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -109,6 +109,15 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -474,7 +483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -642,17 +651,17 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>DEM-001</t>
+          <t>SCI-001</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Decoupage et demolition de pavage / asphalte</t>
+          <t>Sciage de pavage</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D8" s="4">
@@ -666,7 +675,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Secteurs A / raccordements</t>
+          <t>Zone de reprofilage</t>
         </is>
       </c>
       <c r="H8" s="5" t="n"/>
@@ -674,17 +683,17 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>EXC-001</t>
+          <t>DEM-001</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Excavation de tranchee pour reseau pluvial</t>
+          <t>Enlevement de pavage</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="D9" s="4">
@@ -698,7 +707,7 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Tous secteurs</t>
+          <t>Zone de reprofilage / secteurs A</t>
         </is>
       </c>
       <c r="H9" s="5" t="n"/>
@@ -706,17 +715,17 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>EXC-002</t>
+          <t>EXC-001</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Hydro-excavation pour localisation de conduites existantes</t>
+          <t>Excavation de tranchee pour reseau pluvial</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>h</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="D10" s="4">
@@ -730,7 +739,7 @@
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Secteur P-01 / P-02 / raccord Ø1800</t>
+          <t>Tous secteurs</t>
         </is>
       </c>
       <c r="H10" s="5" t="n"/>
@@ -738,17 +747,17 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>CAN-300</t>
+          <t>EXC-002</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Fourniture et pose conduite pluviale DN300</t>
+          <t>Hydro-excavation pour localisation de conduites existantes</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>h</t>
         </is>
       </c>
       <c r="D11" s="4">
@@ -762,7 +771,7 @@
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Schema hydraulique principal</t>
+          <t>Secteur P-01 / P-02 / raccord Ø1800</t>
         </is>
       </c>
       <c r="H11" s="5" t="n"/>
@@ -770,12 +779,12 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>CAN-375</t>
+          <t>CAN-300</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Fourniture et pose raccord / conduite DN375</t>
+          <t>Fourniture et pose conduite pluviale DN300</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -794,7 +803,7 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Raccord propose</t>
+          <t>Secteurs avec conduites nouvelles</t>
         </is>
       </c>
       <c r="H12" s="5" t="n"/>
@@ -802,17 +811,17 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>REG-001</t>
+          <t>CAN-375</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Regard RP-01 (ajustement / reconstruction locale)</t>
+          <t>Fourniture et pose raccord / conduite DN375</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D13" s="4">
@@ -826,7 +835,7 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Noeud de repartition</t>
+          <t>Raccord propose</t>
         </is>
       </c>
       <c r="H13" s="5" t="n"/>
@@ -834,12 +843,12 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>REG-002</t>
+          <t>REG-001</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Regard RP-02 avec clapet anti-retour</t>
+          <t>Regard RP-01 (ajustement / reconstruction locale)</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -858,7 +867,7 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Aval poste de pompage</t>
+          <t>Noeud de repartition</t>
         </is>
       </c>
       <c r="H14" s="5" t="n"/>
@@ -866,12 +875,12 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>SEP-001</t>
+          <t>REG-002</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Unite de traitement type Jellyfish (DP-01)</t>
+          <t>Regard RP-02 avec clapet anti-retour</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -890,7 +899,7 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Branche traitement</t>
+          <t>Aval poste / reseau existant</t>
         </is>
       </c>
       <c r="H15" s="5" t="n"/>
@@ -898,12 +907,12 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>PUI-001</t>
+          <t>SEP-001</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Nouveau puisard</t>
+          <t>Unite de traitement type Jellyfish (DP-01)</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -922,7 +931,7 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Secteur A</t>
+          <t>Branche traitement</t>
         </is>
       </c>
       <c r="H16" s="5" t="n"/>
@@ -930,17 +939,17 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>BOR-001</t>
+          <t>PUI-001</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Saignee dans bordure / raccord de bordure</t>
+          <t>Nouveau puisard</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>u</t>
         </is>
       </c>
       <c r="D17" s="4">
@@ -962,17 +971,17 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>RAC-001</t>
+          <t>BOR-001</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Raccordement a la conduite existante Ø1800</t>
+          <t>Saignee dans bordure / raccord de bordure</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D18" s="4">
@@ -986,7 +995,7 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Secteur P-01 / P-02</t>
+          <t>Secteur A</t>
         </is>
       </c>
       <c r="H18" s="5" t="n"/>
@@ -994,17 +1003,17 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>REM-001</t>
+          <t>BORD-001</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>Remblai compacte et remise en forme</t>
+          <t>Reconstruction de bordure (si requise)</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D19" s="4">
@@ -1018,7 +1027,7 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Tous secteurs</t>
+          <t>Zone de reprofilage</t>
         </is>
       </c>
       <c r="H19" s="5" t="n"/>
@@ -1026,17 +1035,17 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>PAV-001</t>
+          <t>RAC-001</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Reprofilage / reprise de pavage</t>
+          <t>Raccordement a la conduite existante Ø1800</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>u</t>
         </is>
       </c>
       <c r="D20" s="4">
@@ -1050,7 +1059,7 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Secteurs a risque drainage</t>
+          <t>Secteur P-01 / P-02</t>
         </is>
       </c>
       <c r="H20" s="5" t="n"/>
@@ -1058,17 +1067,17 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>ESS-001</t>
+          <t>REM-001</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Essais / verification hydraulique et mise en service</t>
+          <t>Remblai et materiaux granulaires</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="D21" s="4">
@@ -1082,7 +1091,7 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Reseau pluvial</t>
+          <t>Tous secteurs</t>
         </is>
       </c>
       <c r="H21" s="5" t="n"/>
@@ -1090,17 +1099,17 @@
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>DOC-001</t>
+          <t>PAV-001</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Plans finaux / dossier de recollement</t>
+          <t>Reprofilage / reprise de pavage</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="D22" s="4">
@@ -1114,19 +1123,147 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
+          <t>Secteurs a risque drainage</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>REF-001</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Refection des surfaces (gazon, etc.)</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="D23" s="4">
+        <f>SUMIFS(Detail_Image1!$H:$H,Detail_Image1!$C:$C,$A23)+SUMIFS(Detail_Image2!$H:$H,Detail_Image2!$C:$C,$A23)+SUMIFS(Detail_Image3!$H:$H,Detail_Image3!$C:$C,$A23)+SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A23)</f>
+        <v/>
+      </c>
+      <c r="E23" s="4" t="n"/>
+      <c r="F23" s="4">
+        <f>IF(E23="","",D23*E23)</f>
+        <v/>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>Zone de reprofilage / finitions</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>AJU-001</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Ajustement d'ouvrages existants</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+      <c r="D24" s="9">
+        <f>SUMIFS(Detail_Image1!$H:$H,Detail_Image1!$C:$C,$A24)+SUMIFS(Detail_Image2!$H:$H,Detail_Image2!$C:$C,$A24)+SUMIFS(Detail_Image3!$H:$H,Detail_Image3!$C:$C,$A24)+SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A24)</f>
+        <v/>
+      </c>
+      <c r="E24" s="4" t="n"/>
+      <c r="F24" s="9">
+        <f>IF(E24="","",D24*E24)</f>
+        <v/>
+      </c>
+      <c r="G24" s="5" t="inlineStr">
+        <is>
+          <t>Zone de reprofilage / reseau existant</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>ESS-001</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Essais / verification hydraulique et mise en service</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="D25" s="4">
+        <f>SUMIFS(Detail_Image1!$H:$H,Detail_Image1!$C:$C,$A25)+SUMIFS(Detail_Image2!$H:$H,Detail_Image2!$C:$C,$A25)+SUMIFS(Detail_Image3!$H:$H,Detail_Image3!$C:$C,$A25)+SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A25)</f>
+        <v/>
+      </c>
+      <c r="E25" s="4" t="n"/>
+      <c r="F25" s="4">
+        <f>IF(E25="","",D25*E25)</f>
+        <v/>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>Reseau pluvial</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>DOC-001</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Plans finaux / dossier de recollement</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="D26" s="4">
+        <f>SUMIFS(Detail_Image1!$H:$H,Detail_Image1!$C:$C,$A26)+SUMIFS(Detail_Image2!$H:$H,Detail_Image2!$C:$C,$A26)+SUMIFS(Detail_Image3!$H:$H,Detail_Image3!$C:$C,$A26)+SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A26)</f>
+        <v/>
+      </c>
+      <c r="E26" s="4" t="n"/>
+      <c r="F26" s="4">
+        <f>IF(E26="","",D26*E26)</f>
+        <v/>
+      </c>
+      <c r="G26" s="5" t="inlineStr">
+        <is>
           <t>Tous secteurs</t>
         </is>
       </c>
-      <c r="H22" s="5" t="n"/>
-    </row>
-    <row r="24">
-      <c r="D24" s="6" t="inlineStr">
+      <c r="H26" s="5" t="n"/>
+    </row>
+    <row r="28">
+      <c r="D28" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="F24" s="6">
-        <f>SUM(F5:F22)</f>
+      <c r="F28" s="9">
+        <f>SUM(F5:F26)</f>
         <v/>
       </c>
     </row>
@@ -1163,7 +1300,7 @@
     <row r="1">
       <c r="A1" s="7" t="inlineStr">
         <is>
-          <t>Detail quantites - Detail_Image1</t>
+          <t>Detail quantites - Image1 (zone de reprofilage)</t>
         </is>
       </c>
     </row>
@@ -1222,22 +1359,22 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Image1</t>
+          <t>Image1_reprofilage</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Troncon S1</t>
+          <t>Zone de reprofilage</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>CAN-300</t>
+          <t>SCI-001</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Conduite DN300 StormBrixx -&gt; RP-01</t>
+          <t>Sciage de pavage</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -1246,7 +1383,7 @@
         </is>
       </c>
       <c r="F4" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G4" s="4" t="n">
         <v>1</v>
@@ -1257,7 +1394,7 @@
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Mesure lue sur schema hydraulique</t>
+          <t>Longueur a mesurer sur plan DAO/PDF</t>
         </is>
       </c>
       <c r="J4" s="5" t="n"/>
@@ -1265,31 +1402,31 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Image1</t>
+          <t>Image1_reprofilage</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Troncon S2</t>
+          <t>Zone de reprofilage</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>CAN-300</t>
+          <t>DEM-001</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Conduite DN300 RP-01 -&gt; point de convergence</t>
+          <t>Enlevement de pavage</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>7</v>
+        <v>557</v>
       </c>
       <c r="G5" s="4" t="n">
         <v>1</v>
@@ -1300,30 +1437,34 @@
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Mesure lue sur schema hydraulique</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="n"/>
+          <t>Image ajoutee: zone delimitee 557 m2</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr">
+        <is>
+          <t>Hypothese: enlevement sur toute la zone reprise</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>Image1</t>
+          <t>Image1_reprofilage</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Troncon S3</t>
+          <t>Zone de reprofilage</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>CAN-300</t>
+          <t>BORD-001</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Conduite DN300 vers DP-01 (branche derivee)</t>
+          <t>Reconstruction de bordure (si requise)</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -1332,7 +1473,7 @@
         </is>
       </c>
       <c r="F6" s="4" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="G6" s="4" t="n">
         <v>1</v>
@@ -1343,7 +1484,7 @@
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Mesure lue sur schema hydraulique</t>
+          <t>Longueur conditionnelle selon etat existant</t>
         </is>
       </c>
       <c r="J6" s="5" t="n"/>
@@ -1351,31 +1492,31 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Image1</t>
+          <t>Image1_reprofilage</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Troncon S4</t>
+          <t>Zone de reprofilage</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>CAN-300</t>
+          <t>REM-001</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Conduite DN300 retour DP-01 -&gt; convergence</t>
+          <t>Remblai et materiaux granulaires</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="G7" s="4" t="n">
         <v>1</v>
@@ -1386,7 +1527,7 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Mesure a confirmer sur plan IFC</t>
+          <t>Volume apres profils et epaisseur finale</t>
         </is>
       </c>
       <c r="J7" s="5" t="n"/>
@@ -1394,31 +1535,31 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Image1</t>
+          <t>Image1_reprofilage</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Troncon S5</t>
+          <t>Zone de reprofilage</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>CAN-300</t>
+          <t>AJU-001</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Conduite DN300 convergence -&gt; RP-02</t>
+          <t>Ajustement d'ouvrages existants</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>u</t>
         </is>
       </c>
       <c r="F8" s="4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G8" s="4" t="n">
         <v>1</v>
@@ -1429,7 +1570,7 @@
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Mesure lue sur schema hydraulique</t>
+          <t>Minimum 1 unite, ajuster apres releve terrain</t>
         </is>
       </c>
       <c r="J8" s="5" t="n"/>
@@ -1437,31 +1578,31 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Image1</t>
+          <t>Image1_reprofilage</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Troncon S6</t>
+          <t>Zone de reprofilage</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>CAN-300</t>
+          <t>PAV-001</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Conduite DN300 RP-02 -&gt; exutoire gravitaire</t>
+          <t>Reprofilage / reprise de pavage (point bas a elev. 29,720 m)</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>14.5</v>
+        <v>557</v>
       </c>
       <c r="G9" s="4" t="n">
         <v>1</v>
@@ -1472,39 +1613,43 @@
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Mesure lue sur schema hydraulique</t>
-        </is>
-      </c>
-      <c r="J9" s="5" t="n"/>
+          <t>Image ajoutee: annotation 557 m2 + cote 29,720</t>
+        </is>
+      </c>
+      <c r="J9" s="5" t="inlineStr">
+        <is>
+          <t>Surface de reprise de pavage selon zone surlignee</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Image1</t>
+          <t>Image1_reprofilage</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Noeud RP-01</t>
+          <t>Zone de reprofilage</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>REG-001</t>
+          <t>REF-001</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Regard RP-01 regulateur (ajustement/reprise)</t>
+          <t>Refection des surfaces (gazon, etc.)</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="F10" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" s="4" t="n">
         <v>1</v>
@@ -1515,107 +1660,50 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>Quantite minimale = 1</t>
-        </is>
-      </c>
-      <c r="J10" s="5" t="n"/>
+          <t>Si surfaces non pavees sont affectees</t>
+        </is>
+      </c>
+      <c r="J10" s="5" t="inlineStr">
+        <is>
+          <t>A ajuster apres verification terrain</t>
+        </is>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Image1</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Branche traitement</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>SEP-001</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>Unite de traitement type Jellyfish (DP-01)</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>u</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" s="4">
-        <f>IF(F11="","",F11*G11)</f>
-        <v/>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>Valider modele/fournisseur</t>
-        </is>
-      </c>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Sous-total (controle)</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n"/>
+      <c r="C11" s="4" t="n"/>
+      <c r="D11" s="5" t="n"/>
+      <c r="E11" s="4" t="n"/>
+      <c r="F11" s="4" t="n"/>
+      <c r="G11" s="4" t="n"/>
+      <c r="H11" s="11">
+        <f>SUM(H4:H10)</f>
+        <v/>
+      </c>
+      <c r="I11" s="5" t="n"/>
       <c r="J11" s="5" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>Image1</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Aval pompage</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>REG-002</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>Regard RP-02 avec clapet</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>u</t>
-        </is>
-      </c>
-      <c r="F12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" s="4">
-        <f>IF(F12="","",F12*G12)</f>
-        <v/>
-      </c>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>Quantite minimale = 1</t>
-        </is>
-      </c>
+      <c r="A12" s="4" t="n"/>
+      <c r="B12" s="5" t="n"/>
+      <c r="C12" s="4" t="n"/>
+      <c r="D12" s="5" t="n"/>
+      <c r="E12" s="4" t="n"/>
+      <c r="F12" s="4" t="n"/>
+      <c r="G12" s="4" t="n"/>
+      <c r="H12" s="4" t="n"/>
+      <c r="I12" s="5" t="n"/>
       <c r="J12" s="5" t="n"/>
     </row>
+    <row r="13"/>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
-        <is>
-          <t>Sous-total (controle)</t>
-        </is>
-      </c>
-      <c r="H14" s="8">
-        <f>SUM(H4:H12)</f>
-        <v/>
-      </c>
+      <c r="A14" s="8" t="n"/>
+      <c r="H14" s="8" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2530,7 +2618,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -2610,6 +2698,13 @@
       <c r="A13" t="inlineStr">
         <is>
           <t>- Remplacer les hypotheses par metrage DAO/terrain des que disponible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>- Detail_Image1 a ete remplace par la zone de reprofilage (items de preparation/refection) selon la nouvelle image.</t>
         </is>
       </c>
     </row>
@@ -2624,7 +2719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2724,100 +2819,100 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>DEM-001</t>
+          <t>SCI-001</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Decoupage et demolition de pavage / asphalte</t>
+          <t>Sciage de pavage</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>Secteurs A / raccordements</t>
+          <t>Zone de reprofilage</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>EXC-001</t>
+          <t>DEM-001</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Excavation de tranchee pour reseau pluvial</t>
+          <t>Enlevement de pavage</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Tous secteurs</t>
+          <t>Zone de reprofilage / secteurs A</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>EXC-002</t>
+          <t>EXC-001</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>Hydro-excavation pour localisation de conduites existantes</t>
+          <t>Excavation de tranchee pour reseau pluvial</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>h</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Secteur P-01 / P-02 / raccord Ø1800</t>
+          <t>Tous secteurs</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>CAN-300</t>
+          <t>EXC-002</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Fourniture et pose conduite pluviale DN300</t>
+          <t>Hydro-excavation pour localisation de conduites existantes</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>h</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>Schema hydraulique principal</t>
+          <t>Secteur P-01 / P-02 / raccord Ø1800</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>CAN-375</t>
+          <t>CAN-300</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>Fourniture et pose raccord / conduite DN375</t>
+          <t>Fourniture et pose conduite pluviale DN300</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -2827,41 +2922,41 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Raccord propose</t>
+          <t>Secteurs avec conduites nouvelles</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>REG-001</t>
+          <t>CAN-375</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t>Regard RP-01 (ajustement / reconstruction locale)</t>
+          <t>Fourniture et pose raccord / conduite DN375</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Noeud de repartition</t>
+          <t>Raccord propose</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>REG-002</t>
+          <t>REG-001</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Regard RP-02 avec clapet anti-retour</t>
+          <t>Regard RP-01 (ajustement / reconstruction locale)</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
@@ -2871,19 +2966,19 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Aval poste de pompage</t>
+          <t>Noeud de repartition</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>SEP-001</t>
+          <t>REG-002</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Unite de traitement type Jellyfish (DP-01)</t>
+          <t>Regard RP-02 avec clapet anti-retour</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -2893,19 +2988,19 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Branche traitement</t>
+          <t>Aval poste / reseau existant</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>PUI-001</t>
+          <t>SEP-001</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Nouveau puisard</t>
+          <t>Unite de traitement type Jellyfish (DP-01)</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -2915,24 +3010,24 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Secteur A</t>
+          <t>Branche traitement</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>BOR-001</t>
+          <t>PUI-001</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>Saignee dans bordure / raccord de bordure</t>
+          <t>Nouveau puisard</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>u</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -2944,108 +3039,196 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>RAC-001</t>
+          <t>BOR-001</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Raccordement a la conduite existante Ø1800</t>
+          <t>Saignee dans bordure / raccord de bordure</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
         <is>
-          <t>Secteur P-01 / P-02</t>
+          <t>Secteur A</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>REM-001</t>
+          <t>BORD-001</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>Remblai compacte et remise en forme</t>
+          <t>Reconstruction de bordure (si requise)</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>m3</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
         <is>
-          <t>Tous secteurs</t>
+          <t>Zone de reprofilage</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>PAV-001</t>
+          <t>RAC-001</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Reprofilage / reprise de pavage</t>
+          <t>Raccordement a la conduite existante Ø1800</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>u</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Secteurs a risque drainage</t>
+          <t>Secteur P-01 / P-02</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>ESS-001</t>
+          <t>REM-001</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>Essais / verification hydraulique et mise en service</t>
+          <t>Remblai et materiaux granulaires</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>lot</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Reseau pluvial</t>
+          <t>Tous secteurs</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
+          <t>PAV-001</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Reprofilage / reprise de pavage</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>Secteurs a risque drainage</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>REF-001</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Refection des surfaces (gazon, etc.)</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>m2</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>Zone de reprofilage / finitions</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>AJU-001</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Ajustement d'ouvrages existants</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>Zone de reprofilage / reseau existant</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>ESS-001</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Essais / verification hydraulique et mise en service</t>
+        </is>
+      </c>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>lot</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Reseau pluvial</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
           <t>DOC-001</t>
         </is>
       </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="B23" s="5" t="inlineStr">
         <is>
           <t>Plans finaux / dossier de recollement</t>
         </is>
       </c>
-      <c r="C19" s="4" t="inlineStr">
+      <c r="C23" s="4" t="inlineStr">
         <is>
           <t>lot</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>Tous secteurs</t>
         </is>

</xml_diff>

<commit_message>
Add per-sector cost estimation tab to BOQ workbook
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/Bordereau_prix_drainage_par_secteur.xlsx
+++ b/engineering/stormwater-pumping/Bordereau_prix_drainage_par_secteur.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Detail_facade_batim" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Traceabilite" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Catalogue_items" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Estimation_par_secteur" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -75,8 +76,19 @@
       <b val="1"/>
       <sz val="13"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -95,8 +107,18 @@
         <bgColor rgb="FFCCFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -119,6 +141,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -130,7 +166,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -209,6 +245,35 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -3328,4 +3393,1352 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" style="14" min="1" max="1"/>
+    <col width="48" customWidth="1" style="14" min="2" max="2"/>
+    <col width="10" customWidth="1" style="14" min="3" max="3"/>
+    <col width="12" customWidth="1" style="14" min="4" max="4"/>
+    <col width="12" customWidth="1" style="14" min="5" max="5"/>
+    <col width="12" customWidth="1" style="14" min="6" max="6"/>
+    <col width="12" customWidth="1" style="14" min="7" max="7"/>
+    <col width="12" customWidth="1" style="14" min="8" max="8"/>
+    <col width="14" customWidth="1" style="14" min="9" max="9"/>
+    <col width="14" customWidth="1" style="14" min="10" max="10"/>
+    <col width="18" customWidth="1" style="14" min="11" max="11"/>
+    <col width="18" customWidth="1" style="14" min="12" max="12"/>
+    <col width="14" customWidth="1" style="14" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>ESTIMATION DES COUTS PAR SECTEUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>Synthese des couts par secteur (CAD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>Secteur A</t>
+        </is>
+      </c>
+      <c r="B4" s="30">
+        <f>SUM(F13:F33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>Secteur P</t>
+        </is>
+      </c>
+      <c r="B5" s="30">
+        <f>SUM(H13:H33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>Façade (reseau)</t>
+        </is>
+      </c>
+      <c r="B6" s="30">
+        <f>SUM(J13:J33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>Façade (topo/doc)</t>
+        </is>
+      </c>
+      <c r="B7" s="30">
+        <f>SUM(L13:L33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="31" t="inlineStr">
+        <is>
+          <t>TOTAL GENERAL</t>
+        </is>
+      </c>
+      <c r="B8" s="32">
+        <f>SUM(B4:B7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>Controle vs Bordereau_prix</t>
+        </is>
+      </c>
+      <c r="B9" s="34">
+        <f>B8-Bordereau_prix!F27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="35" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B12" s="35" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C12" s="35" t="inlineStr">
+        <is>
+          <t>Unite</t>
+        </is>
+      </c>
+      <c r="D12" s="35" t="inlineStr">
+        <is>
+          <t>PU</t>
+        </is>
+      </c>
+      <c r="E12" s="35" t="inlineStr">
+        <is>
+          <t>Qte_A</t>
+        </is>
+      </c>
+      <c r="F12" s="35" t="inlineStr">
+        <is>
+          <t>Cout_A</t>
+        </is>
+      </c>
+      <c r="G12" s="35" t="inlineStr">
+        <is>
+          <t>Qte_P</t>
+        </is>
+      </c>
+      <c r="H12" s="35" t="inlineStr">
+        <is>
+          <t>Cout_P</t>
+        </is>
+      </c>
+      <c r="I12" s="35" t="inlineStr">
+        <is>
+          <t>Qte_Facade</t>
+        </is>
+      </c>
+      <c r="J12" s="35" t="inlineStr">
+        <is>
+          <t>Cout_Facade</t>
+        </is>
+      </c>
+      <c r="K12" s="35" t="inlineStr">
+        <is>
+          <t>Qte_Facade_detail</t>
+        </is>
+      </c>
+      <c r="L12" s="35" t="inlineStr">
+        <is>
+          <t>Cout_Facade_detail</t>
+        </is>
+      </c>
+      <c r="M12" s="35" t="inlineStr">
+        <is>
+          <t>Cout_total_item</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="36">
+        <f>Bordereau_prix!A5</f>
+        <v/>
+      </c>
+      <c r="B13" s="37">
+        <f>Bordereau_prix!B5</f>
+        <v/>
+      </c>
+      <c r="C13" s="36">
+        <f>Bordereau_prix!C5</f>
+        <v/>
+      </c>
+      <c r="D13" s="36">
+        <f>Bordereau_prix!E5</f>
+        <v/>
+      </c>
+      <c r="E13" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A13)</f>
+        <v/>
+      </c>
+      <c r="F13" s="36">
+        <f>E13*D13</f>
+        <v/>
+      </c>
+      <c r="G13" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A13)</f>
+        <v/>
+      </c>
+      <c r="H13" s="36">
+        <f>G13*D13</f>
+        <v/>
+      </c>
+      <c r="I13" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A13)</f>
+        <v/>
+      </c>
+      <c r="J13" s="36">
+        <f>I13*D13</f>
+        <v/>
+      </c>
+      <c r="K13" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A13)</f>
+        <v/>
+      </c>
+      <c r="L13" s="36">
+        <f>K13*D13</f>
+        <v/>
+      </c>
+      <c r="M13" s="36">
+        <f>SUM(F13,H13,J13,L13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="36">
+        <f>Bordereau_prix!A6</f>
+        <v/>
+      </c>
+      <c r="B14" s="37">
+        <f>Bordereau_prix!B6</f>
+        <v/>
+      </c>
+      <c r="C14" s="36">
+        <f>Bordereau_prix!C6</f>
+        <v/>
+      </c>
+      <c r="D14" s="36">
+        <f>Bordereau_prix!E6</f>
+        <v/>
+      </c>
+      <c r="E14" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A14)</f>
+        <v/>
+      </c>
+      <c r="F14" s="36">
+        <f>E14*D14</f>
+        <v/>
+      </c>
+      <c r="G14" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A14)</f>
+        <v/>
+      </c>
+      <c r="H14" s="36">
+        <f>G14*D14</f>
+        <v/>
+      </c>
+      <c r="I14" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A14)</f>
+        <v/>
+      </c>
+      <c r="J14" s="36">
+        <f>I14*D14</f>
+        <v/>
+      </c>
+      <c r="K14" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A14)</f>
+        <v/>
+      </c>
+      <c r="L14" s="36">
+        <f>K14*D14</f>
+        <v/>
+      </c>
+      <c r="M14" s="36">
+        <f>SUM(F14,H14,J14,L14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="36">
+        <f>Bordereau_prix!A7</f>
+        <v/>
+      </c>
+      <c r="B15" s="37">
+        <f>Bordereau_prix!B7</f>
+        <v/>
+      </c>
+      <c r="C15" s="36">
+        <f>Bordereau_prix!C7</f>
+        <v/>
+      </c>
+      <c r="D15" s="36">
+        <f>Bordereau_prix!E7</f>
+        <v/>
+      </c>
+      <c r="E15" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A15)</f>
+        <v/>
+      </c>
+      <c r="F15" s="36">
+        <f>E15*D15</f>
+        <v/>
+      </c>
+      <c r="G15" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A15)</f>
+        <v/>
+      </c>
+      <c r="H15" s="36">
+        <f>G15*D15</f>
+        <v/>
+      </c>
+      <c r="I15" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A15)</f>
+        <v/>
+      </c>
+      <c r="J15" s="36">
+        <f>I15*D15</f>
+        <v/>
+      </c>
+      <c r="K15" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A15)</f>
+        <v/>
+      </c>
+      <c r="L15" s="36">
+        <f>K15*D15</f>
+        <v/>
+      </c>
+      <c r="M15" s="36">
+        <f>SUM(F15,H15,J15,L15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="36">
+        <f>Bordereau_prix!A8</f>
+        <v/>
+      </c>
+      <c r="B16" s="37">
+        <f>Bordereau_prix!B8</f>
+        <v/>
+      </c>
+      <c r="C16" s="36">
+        <f>Bordereau_prix!C8</f>
+        <v/>
+      </c>
+      <c r="D16" s="36">
+        <f>Bordereau_prix!E8</f>
+        <v/>
+      </c>
+      <c r="E16" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A16)</f>
+        <v/>
+      </c>
+      <c r="F16" s="36">
+        <f>E16*D16</f>
+        <v/>
+      </c>
+      <c r="G16" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A16)</f>
+        <v/>
+      </c>
+      <c r="H16" s="36">
+        <f>G16*D16</f>
+        <v/>
+      </c>
+      <c r="I16" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A16)</f>
+        <v/>
+      </c>
+      <c r="J16" s="36">
+        <f>I16*D16</f>
+        <v/>
+      </c>
+      <c r="K16" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A16)</f>
+        <v/>
+      </c>
+      <c r="L16" s="36">
+        <f>K16*D16</f>
+        <v/>
+      </c>
+      <c r="M16" s="36">
+        <f>SUM(F16,H16,J16,L16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="36">
+        <f>Bordereau_prix!A9</f>
+        <v/>
+      </c>
+      <c r="B17" s="37">
+        <f>Bordereau_prix!B9</f>
+        <v/>
+      </c>
+      <c r="C17" s="36">
+        <f>Bordereau_prix!C9</f>
+        <v/>
+      </c>
+      <c r="D17" s="36">
+        <f>Bordereau_prix!E9</f>
+        <v/>
+      </c>
+      <c r="E17" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A17)</f>
+        <v/>
+      </c>
+      <c r="F17" s="36">
+        <f>E17*D17</f>
+        <v/>
+      </c>
+      <c r="G17" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A17)</f>
+        <v/>
+      </c>
+      <c r="H17" s="36">
+        <f>G17*D17</f>
+        <v/>
+      </c>
+      <c r="I17" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A17)</f>
+        <v/>
+      </c>
+      <c r="J17" s="36">
+        <f>I17*D17</f>
+        <v/>
+      </c>
+      <c r="K17" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A17)</f>
+        <v/>
+      </c>
+      <c r="L17" s="36">
+        <f>K17*D17</f>
+        <v/>
+      </c>
+      <c r="M17" s="36">
+        <f>SUM(F17,H17,J17,L17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="36">
+        <f>Bordereau_prix!A10</f>
+        <v/>
+      </c>
+      <c r="B18" s="37">
+        <f>Bordereau_prix!B10</f>
+        <v/>
+      </c>
+      <c r="C18" s="36">
+        <f>Bordereau_prix!C10</f>
+        <v/>
+      </c>
+      <c r="D18" s="36">
+        <f>Bordereau_prix!E10</f>
+        <v/>
+      </c>
+      <c r="E18" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A18)</f>
+        <v/>
+      </c>
+      <c r="F18" s="36">
+        <f>E18*D18</f>
+        <v/>
+      </c>
+      <c r="G18" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A18)</f>
+        <v/>
+      </c>
+      <c r="H18" s="36">
+        <f>G18*D18</f>
+        <v/>
+      </c>
+      <c r="I18" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A18)</f>
+        <v/>
+      </c>
+      <c r="J18" s="36">
+        <f>I18*D18</f>
+        <v/>
+      </c>
+      <c r="K18" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A18)</f>
+        <v/>
+      </c>
+      <c r="L18" s="36">
+        <f>K18*D18</f>
+        <v/>
+      </c>
+      <c r="M18" s="36">
+        <f>SUM(F18,H18,J18,L18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="36">
+        <f>Bordereau_prix!A11</f>
+        <v/>
+      </c>
+      <c r="B19" s="37">
+        <f>Bordereau_prix!B11</f>
+        <v/>
+      </c>
+      <c r="C19" s="36">
+        <f>Bordereau_prix!C11</f>
+        <v/>
+      </c>
+      <c r="D19" s="36">
+        <f>Bordereau_prix!E11</f>
+        <v/>
+      </c>
+      <c r="E19" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A19)</f>
+        <v/>
+      </c>
+      <c r="F19" s="36">
+        <f>E19*D19</f>
+        <v/>
+      </c>
+      <c r="G19" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A19)</f>
+        <v/>
+      </c>
+      <c r="H19" s="36">
+        <f>G19*D19</f>
+        <v/>
+      </c>
+      <c r="I19" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A19)</f>
+        <v/>
+      </c>
+      <c r="J19" s="36">
+        <f>I19*D19</f>
+        <v/>
+      </c>
+      <c r="K19" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A19)</f>
+        <v/>
+      </c>
+      <c r="L19" s="36">
+        <f>K19*D19</f>
+        <v/>
+      </c>
+      <c r="M19" s="36">
+        <f>SUM(F19,H19,J19,L19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="36">
+        <f>Bordereau_prix!A12</f>
+        <v/>
+      </c>
+      <c r="B20" s="37">
+        <f>Bordereau_prix!B12</f>
+        <v/>
+      </c>
+      <c r="C20" s="36">
+        <f>Bordereau_prix!C12</f>
+        <v/>
+      </c>
+      <c r="D20" s="36">
+        <f>Bordereau_prix!E12</f>
+        <v/>
+      </c>
+      <c r="E20" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A20)</f>
+        <v/>
+      </c>
+      <c r="F20" s="36">
+        <f>E20*D20</f>
+        <v/>
+      </c>
+      <c r="G20" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A20)</f>
+        <v/>
+      </c>
+      <c r="H20" s="36">
+        <f>G20*D20</f>
+        <v/>
+      </c>
+      <c r="I20" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A20)</f>
+        <v/>
+      </c>
+      <c r="J20" s="36">
+        <f>I20*D20</f>
+        <v/>
+      </c>
+      <c r="K20" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A20)</f>
+        <v/>
+      </c>
+      <c r="L20" s="36">
+        <f>K20*D20</f>
+        <v/>
+      </c>
+      <c r="M20" s="36">
+        <f>SUM(F20,H20,J20,L20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="36">
+        <f>Bordereau_prix!A13</f>
+        <v/>
+      </c>
+      <c r="B21" s="37">
+        <f>Bordereau_prix!B13</f>
+        <v/>
+      </c>
+      <c r="C21" s="36">
+        <f>Bordereau_prix!C13</f>
+        <v/>
+      </c>
+      <c r="D21" s="36">
+        <f>Bordereau_prix!E13</f>
+        <v/>
+      </c>
+      <c r="E21" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A21)</f>
+        <v/>
+      </c>
+      <c r="F21" s="36">
+        <f>E21*D21</f>
+        <v/>
+      </c>
+      <c r="G21" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A21)</f>
+        <v/>
+      </c>
+      <c r="H21" s="36">
+        <f>G21*D21</f>
+        <v/>
+      </c>
+      <c r="I21" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A21)</f>
+        <v/>
+      </c>
+      <c r="J21" s="36">
+        <f>I21*D21</f>
+        <v/>
+      </c>
+      <c r="K21" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A21)</f>
+        <v/>
+      </c>
+      <c r="L21" s="36">
+        <f>K21*D21</f>
+        <v/>
+      </c>
+      <c r="M21" s="36">
+        <f>SUM(F21,H21,J21,L21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="36">
+        <f>Bordereau_prix!A14</f>
+        <v/>
+      </c>
+      <c r="B22" s="37">
+        <f>Bordereau_prix!B14</f>
+        <v/>
+      </c>
+      <c r="C22" s="36">
+        <f>Bordereau_prix!C14</f>
+        <v/>
+      </c>
+      <c r="D22" s="36">
+        <f>Bordereau_prix!E14</f>
+        <v/>
+      </c>
+      <c r="E22" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A22)</f>
+        <v/>
+      </c>
+      <c r="F22" s="36">
+        <f>E22*D22</f>
+        <v/>
+      </c>
+      <c r="G22" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A22)</f>
+        <v/>
+      </c>
+      <c r="H22" s="36">
+        <f>G22*D22</f>
+        <v/>
+      </c>
+      <c r="I22" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A22)</f>
+        <v/>
+      </c>
+      <c r="J22" s="36">
+        <f>I22*D22</f>
+        <v/>
+      </c>
+      <c r="K22" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A22)</f>
+        <v/>
+      </c>
+      <c r="L22" s="36">
+        <f>K22*D22</f>
+        <v/>
+      </c>
+      <c r="M22" s="36">
+        <f>SUM(F22,H22,J22,L22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="36">
+        <f>Bordereau_prix!A15</f>
+        <v/>
+      </c>
+      <c r="B23" s="37">
+        <f>Bordereau_prix!B15</f>
+        <v/>
+      </c>
+      <c r="C23" s="36">
+        <f>Bordereau_prix!C15</f>
+        <v/>
+      </c>
+      <c r="D23" s="36">
+        <f>Bordereau_prix!E15</f>
+        <v/>
+      </c>
+      <c r="E23" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A23)</f>
+        <v/>
+      </c>
+      <c r="F23" s="36">
+        <f>E23*D23</f>
+        <v/>
+      </c>
+      <c r="G23" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A23)</f>
+        <v/>
+      </c>
+      <c r="H23" s="36">
+        <f>G23*D23</f>
+        <v/>
+      </c>
+      <c r="I23" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A23)</f>
+        <v/>
+      </c>
+      <c r="J23" s="36">
+        <f>I23*D23</f>
+        <v/>
+      </c>
+      <c r="K23" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A23)</f>
+        <v/>
+      </c>
+      <c r="L23" s="36">
+        <f>K23*D23</f>
+        <v/>
+      </c>
+      <c r="M23" s="36">
+        <f>SUM(F23,H23,J23,L23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="36">
+        <f>Bordereau_prix!A16</f>
+        <v/>
+      </c>
+      <c r="B24" s="37">
+        <f>Bordereau_prix!B16</f>
+        <v/>
+      </c>
+      <c r="C24" s="36">
+        <f>Bordereau_prix!C16</f>
+        <v/>
+      </c>
+      <c r="D24" s="36">
+        <f>Bordereau_prix!E16</f>
+        <v/>
+      </c>
+      <c r="E24" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A24)</f>
+        <v/>
+      </c>
+      <c r="F24" s="36">
+        <f>E24*D24</f>
+        <v/>
+      </c>
+      <c r="G24" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A24)</f>
+        <v/>
+      </c>
+      <c r="H24" s="36">
+        <f>G24*D24</f>
+        <v/>
+      </c>
+      <c r="I24" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A24)</f>
+        <v/>
+      </c>
+      <c r="J24" s="36">
+        <f>I24*D24</f>
+        <v/>
+      </c>
+      <c r="K24" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A24)</f>
+        <v/>
+      </c>
+      <c r="L24" s="36">
+        <f>K24*D24</f>
+        <v/>
+      </c>
+      <c r="M24" s="36">
+        <f>SUM(F24,H24,J24,L24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="36">
+        <f>Bordereau_prix!A17</f>
+        <v/>
+      </c>
+      <c r="B25" s="37">
+        <f>Bordereau_prix!B17</f>
+        <v/>
+      </c>
+      <c r="C25" s="36">
+        <f>Bordereau_prix!C17</f>
+        <v/>
+      </c>
+      <c r="D25" s="36">
+        <f>Bordereau_prix!E17</f>
+        <v/>
+      </c>
+      <c r="E25" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A25)</f>
+        <v/>
+      </c>
+      <c r="F25" s="36">
+        <f>E25*D25</f>
+        <v/>
+      </c>
+      <c r="G25" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A25)</f>
+        <v/>
+      </c>
+      <c r="H25" s="36">
+        <f>G25*D25</f>
+        <v/>
+      </c>
+      <c r="I25" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A25)</f>
+        <v/>
+      </c>
+      <c r="J25" s="36">
+        <f>I25*D25</f>
+        <v/>
+      </c>
+      <c r="K25" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A25)</f>
+        <v/>
+      </c>
+      <c r="L25" s="36">
+        <f>K25*D25</f>
+        <v/>
+      </c>
+      <c r="M25" s="36">
+        <f>SUM(F25,H25,J25,L25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="36">
+        <f>Bordereau_prix!A18</f>
+        <v/>
+      </c>
+      <c r="B26" s="37">
+        <f>Bordereau_prix!B18</f>
+        <v/>
+      </c>
+      <c r="C26" s="36">
+        <f>Bordereau_prix!C18</f>
+        <v/>
+      </c>
+      <c r="D26" s="36">
+        <f>Bordereau_prix!E18</f>
+        <v/>
+      </c>
+      <c r="E26" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A26)</f>
+        <v/>
+      </c>
+      <c r="F26" s="36">
+        <f>E26*D26</f>
+        <v/>
+      </c>
+      <c r="G26" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A26)</f>
+        <v/>
+      </c>
+      <c r="H26" s="36">
+        <f>G26*D26</f>
+        <v/>
+      </c>
+      <c r="I26" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A26)</f>
+        <v/>
+      </c>
+      <c r="J26" s="36">
+        <f>I26*D26</f>
+        <v/>
+      </c>
+      <c r="K26" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A26)</f>
+        <v/>
+      </c>
+      <c r="L26" s="36">
+        <f>K26*D26</f>
+        <v/>
+      </c>
+      <c r="M26" s="36">
+        <f>SUM(F26,H26,J26,L26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="36">
+        <f>Bordereau_prix!A19</f>
+        <v/>
+      </c>
+      <c r="B27" s="37">
+        <f>Bordereau_prix!B19</f>
+        <v/>
+      </c>
+      <c r="C27" s="36">
+        <f>Bordereau_prix!C19</f>
+        <v/>
+      </c>
+      <c r="D27" s="36">
+        <f>Bordereau_prix!E19</f>
+        <v/>
+      </c>
+      <c r="E27" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A27)</f>
+        <v/>
+      </c>
+      <c r="F27" s="36">
+        <f>E27*D27</f>
+        <v/>
+      </c>
+      <c r="G27" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A27)</f>
+        <v/>
+      </c>
+      <c r="H27" s="36">
+        <f>G27*D27</f>
+        <v/>
+      </c>
+      <c r="I27" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A27)</f>
+        <v/>
+      </c>
+      <c r="J27" s="36">
+        <f>I27*D27</f>
+        <v/>
+      </c>
+      <c r="K27" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A27)</f>
+        <v/>
+      </c>
+      <c r="L27" s="36">
+        <f>K27*D27</f>
+        <v/>
+      </c>
+      <c r="M27" s="36">
+        <f>SUM(F27,H27,J27,L27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="36">
+        <f>Bordereau_prix!A20</f>
+        <v/>
+      </c>
+      <c r="B28" s="37">
+        <f>Bordereau_prix!B20</f>
+        <v/>
+      </c>
+      <c r="C28" s="36">
+        <f>Bordereau_prix!C20</f>
+        <v/>
+      </c>
+      <c r="D28" s="36">
+        <f>Bordereau_prix!E20</f>
+        <v/>
+      </c>
+      <c r="E28" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A28)</f>
+        <v/>
+      </c>
+      <c r="F28" s="36">
+        <f>E28*D28</f>
+        <v/>
+      </c>
+      <c r="G28" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A28)</f>
+        <v/>
+      </c>
+      <c r="H28" s="36">
+        <f>G28*D28</f>
+        <v/>
+      </c>
+      <c r="I28" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A28)</f>
+        <v/>
+      </c>
+      <c r="J28" s="36">
+        <f>I28*D28</f>
+        <v/>
+      </c>
+      <c r="K28" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A28)</f>
+        <v/>
+      </c>
+      <c r="L28" s="36">
+        <f>K28*D28</f>
+        <v/>
+      </c>
+      <c r="M28" s="36">
+        <f>SUM(F28,H28,J28,L28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="36">
+        <f>Bordereau_prix!A21</f>
+        <v/>
+      </c>
+      <c r="B29" s="37">
+        <f>Bordereau_prix!B21</f>
+        <v/>
+      </c>
+      <c r="C29" s="36">
+        <f>Bordereau_prix!C21</f>
+        <v/>
+      </c>
+      <c r="D29" s="36">
+        <f>Bordereau_prix!E21</f>
+        <v/>
+      </c>
+      <c r="E29" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A29)</f>
+        <v/>
+      </c>
+      <c r="F29" s="36">
+        <f>E29*D29</f>
+        <v/>
+      </c>
+      <c r="G29" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A29)</f>
+        <v/>
+      </c>
+      <c r="H29" s="36">
+        <f>G29*D29</f>
+        <v/>
+      </c>
+      <c r="I29" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A29)</f>
+        <v/>
+      </c>
+      <c r="J29" s="36">
+        <f>I29*D29</f>
+        <v/>
+      </c>
+      <c r="K29" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A29)</f>
+        <v/>
+      </c>
+      <c r="L29" s="36">
+        <f>K29*D29</f>
+        <v/>
+      </c>
+      <c r="M29" s="36">
+        <f>SUM(F29,H29,J29,L29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="36">
+        <f>Bordereau_prix!A22</f>
+        <v/>
+      </c>
+      <c r="B30" s="37">
+        <f>Bordereau_prix!B22</f>
+        <v/>
+      </c>
+      <c r="C30" s="36">
+        <f>Bordereau_prix!C22</f>
+        <v/>
+      </c>
+      <c r="D30" s="36">
+        <f>Bordereau_prix!E22</f>
+        <v/>
+      </c>
+      <c r="E30" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A30)</f>
+        <v/>
+      </c>
+      <c r="F30" s="36">
+        <f>E30*D30</f>
+        <v/>
+      </c>
+      <c r="G30" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A30)</f>
+        <v/>
+      </c>
+      <c r="H30" s="36">
+        <f>G30*D30</f>
+        <v/>
+      </c>
+      <c r="I30" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A30)</f>
+        <v/>
+      </c>
+      <c r="J30" s="36">
+        <f>I30*D30</f>
+        <v/>
+      </c>
+      <c r="K30" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A30)</f>
+        <v/>
+      </c>
+      <c r="L30" s="36">
+        <f>K30*D30</f>
+        <v/>
+      </c>
+      <c r="M30" s="36">
+        <f>SUM(F30,H30,J30,L30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="36">
+        <f>Bordereau_prix!A23</f>
+        <v/>
+      </c>
+      <c r="B31" s="37">
+        <f>Bordereau_prix!B23</f>
+        <v/>
+      </c>
+      <c r="C31" s="36">
+        <f>Bordereau_prix!C23</f>
+        <v/>
+      </c>
+      <c r="D31" s="36">
+        <f>Bordereau_prix!E23</f>
+        <v/>
+      </c>
+      <c r="E31" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A31)</f>
+        <v/>
+      </c>
+      <c r="F31" s="36">
+        <f>E31*D31</f>
+        <v/>
+      </c>
+      <c r="G31" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A31)</f>
+        <v/>
+      </c>
+      <c r="H31" s="36">
+        <f>G31*D31</f>
+        <v/>
+      </c>
+      <c r="I31" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A31)</f>
+        <v/>
+      </c>
+      <c r="J31" s="36">
+        <f>I31*D31</f>
+        <v/>
+      </c>
+      <c r="K31" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A31)</f>
+        <v/>
+      </c>
+      <c r="L31" s="36">
+        <f>K31*D31</f>
+        <v/>
+      </c>
+      <c r="M31" s="36">
+        <f>SUM(F31,H31,J31,L31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="36">
+        <f>Bordereau_prix!A24</f>
+        <v/>
+      </c>
+      <c r="B32" s="37">
+        <f>Bordereau_prix!B24</f>
+        <v/>
+      </c>
+      <c r="C32" s="36">
+        <f>Bordereau_prix!C24</f>
+        <v/>
+      </c>
+      <c r="D32" s="36">
+        <f>Bordereau_prix!E24</f>
+        <v/>
+      </c>
+      <c r="E32" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A32)</f>
+        <v/>
+      </c>
+      <c r="F32" s="36">
+        <f>E32*D32</f>
+        <v/>
+      </c>
+      <c r="G32" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A32)</f>
+        <v/>
+      </c>
+      <c r="H32" s="36">
+        <f>G32*D32</f>
+        <v/>
+      </c>
+      <c r="I32" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A32)</f>
+        <v/>
+      </c>
+      <c r="J32" s="36">
+        <f>I32*D32</f>
+        <v/>
+      </c>
+      <c r="K32" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A32)</f>
+        <v/>
+      </c>
+      <c r="L32" s="36">
+        <f>K32*D32</f>
+        <v/>
+      </c>
+      <c r="M32" s="36">
+        <f>SUM(F32,H32,J32,L32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="36">
+        <f>Bordereau_prix!A25</f>
+        <v/>
+      </c>
+      <c r="B33" s="37">
+        <f>Bordereau_prix!B25</f>
+        <v/>
+      </c>
+      <c r="C33" s="36">
+        <f>Bordereau_prix!C25</f>
+        <v/>
+      </c>
+      <c r="D33" s="36">
+        <f>Bordereau_prix!E25</f>
+        <v/>
+      </c>
+      <c r="E33" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A33)</f>
+        <v/>
+      </c>
+      <c r="F33" s="36">
+        <f>E33*D33</f>
+        <v/>
+      </c>
+      <c r="G33" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A33)</f>
+        <v/>
+      </c>
+      <c r="H33" s="36">
+        <f>G33*D33</f>
+        <v/>
+      </c>
+      <c r="I33" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A33)</f>
+        <v/>
+      </c>
+      <c r="J33" s="36">
+        <f>I33*D33</f>
+        <v/>
+      </c>
+      <c r="K33" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A33)</f>
+        <v/>
+      </c>
+      <c r="L33" s="36">
+        <f>K33*D33</f>
+        <v/>
+      </c>
+      <c r="M33" s="36">
+        <f>SUM(F33,H33,J33,L33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="32" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="F34" s="32">
+        <f>SUM(F13:F33)</f>
+        <v/>
+      </c>
+      <c r="H34" s="32">
+        <f>SUM(H13:H33)</f>
+        <v/>
+      </c>
+      <c r="J34" s="32">
+        <f>SUM(J13:J33)</f>
+        <v/>
+      </c>
+      <c r="L34" s="32">
+        <f>SUM(L13:L33)</f>
+        <v/>
+      </c>
+      <c r="M34" s="32">
+        <f>SUM(M13:M33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
+        <is>
+          <t>Note: cette feuille conserve la synthese globale et detaille la repartition des couts par secteur.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A36:M36"/>
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
add per-sector estimation tab
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/Bordereau_prix_drainage_par_secteur.xlsx
+++ b/engineering/stormwater-pumping/Bordereau_prix_drainage_par_secteur.xlsx
@@ -14,6 +14,7 @@
     <sheet name="Detail_facade_batim" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Traceabilite" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Catalogue_items" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Estimation_par_secteur" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -23,7 +24,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -75,8 +76,19 @@
       <b val="1"/>
       <sz val="13"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -95,8 +107,18 @@
         <bgColor rgb="FFCCFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -119,6 +141,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -130,7 +166,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -209,6 +245,35 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -3328,4 +3393,1352 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="1" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M36"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" style="14" min="1" max="1"/>
+    <col width="48" customWidth="1" style="14" min="2" max="2"/>
+    <col width="10" customWidth="1" style="14" min="3" max="3"/>
+    <col width="12" customWidth="1" style="14" min="4" max="4"/>
+    <col width="12" customWidth="1" style="14" min="5" max="5"/>
+    <col width="12" customWidth="1" style="14" min="6" max="6"/>
+    <col width="12" customWidth="1" style="14" min="7" max="7"/>
+    <col width="12" customWidth="1" style="14" min="8" max="8"/>
+    <col width="14" customWidth="1" style="14" min="9" max="9"/>
+    <col width="14" customWidth="1" style="14" min="10" max="10"/>
+    <col width="18" customWidth="1" style="14" min="11" max="11"/>
+    <col width="18" customWidth="1" style="14" min="12" max="12"/>
+    <col width="14" customWidth="1" style="14" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>ESTIMATION DES COUTS PAR SECTEUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>Synthese des couts par secteur (CAD)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t>Secteur A</t>
+        </is>
+      </c>
+      <c r="B4" s="30">
+        <f>SUM(F13:F33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="29" t="inlineStr">
+        <is>
+          <t>Secteur P</t>
+        </is>
+      </c>
+      <c r="B5" s="30">
+        <f>SUM(H13:H33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="29" t="inlineStr">
+        <is>
+          <t>Façade (reseau)</t>
+        </is>
+      </c>
+      <c r="B6" s="30">
+        <f>SUM(J13:J33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="29" t="inlineStr">
+        <is>
+          <t>Façade (topo/doc)</t>
+        </is>
+      </c>
+      <c r="B7" s="30">
+        <f>SUM(L13:L33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="31" t="inlineStr">
+        <is>
+          <t>TOTAL GENERAL</t>
+        </is>
+      </c>
+      <c r="B8" s="32">
+        <f>SUM(B4:B7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="33" t="inlineStr">
+        <is>
+          <t>Controle vs Bordereau_prix</t>
+        </is>
+      </c>
+      <c r="B9" s="34">
+        <f>B8-Bordereau_prix!F27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="35" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="B12" s="35" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C12" s="35" t="inlineStr">
+        <is>
+          <t>Unite</t>
+        </is>
+      </c>
+      <c r="D12" s="35" t="inlineStr">
+        <is>
+          <t>PU</t>
+        </is>
+      </c>
+      <c r="E12" s="35" t="inlineStr">
+        <is>
+          <t>Qte_A</t>
+        </is>
+      </c>
+      <c r="F12" s="35" t="inlineStr">
+        <is>
+          <t>Cout_A</t>
+        </is>
+      </c>
+      <c r="G12" s="35" t="inlineStr">
+        <is>
+          <t>Qte_P</t>
+        </is>
+      </c>
+      <c r="H12" s="35" t="inlineStr">
+        <is>
+          <t>Cout_P</t>
+        </is>
+      </c>
+      <c r="I12" s="35" t="inlineStr">
+        <is>
+          <t>Qte_Facade</t>
+        </is>
+      </c>
+      <c r="J12" s="35" t="inlineStr">
+        <is>
+          <t>Cout_Facade</t>
+        </is>
+      </c>
+      <c r="K12" s="35" t="inlineStr">
+        <is>
+          <t>Qte_Facade_detail</t>
+        </is>
+      </c>
+      <c r="L12" s="35" t="inlineStr">
+        <is>
+          <t>Cout_Facade_detail</t>
+        </is>
+      </c>
+      <c r="M12" s="35" t="inlineStr">
+        <is>
+          <t>Cout_total_item</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="36">
+        <f>Bordereau_prix!A5</f>
+        <v/>
+      </c>
+      <c r="B13" s="37">
+        <f>Bordereau_prix!B5</f>
+        <v/>
+      </c>
+      <c r="C13" s="36">
+        <f>Bordereau_prix!C5</f>
+        <v/>
+      </c>
+      <c r="D13" s="36">
+        <f>Bordereau_prix!E5</f>
+        <v/>
+      </c>
+      <c r="E13" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A13)</f>
+        <v/>
+      </c>
+      <c r="F13" s="36">
+        <f>E13*D13</f>
+        <v/>
+      </c>
+      <c r="G13" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A13)</f>
+        <v/>
+      </c>
+      <c r="H13" s="36">
+        <f>G13*D13</f>
+        <v/>
+      </c>
+      <c r="I13" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A13)</f>
+        <v/>
+      </c>
+      <c r="J13" s="36">
+        <f>I13*D13</f>
+        <v/>
+      </c>
+      <c r="K13" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A13)</f>
+        <v/>
+      </c>
+      <c r="L13" s="36">
+        <f>K13*D13</f>
+        <v/>
+      </c>
+      <c r="M13" s="36">
+        <f>SUM(F13,H13,J13,L13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="36">
+        <f>Bordereau_prix!A6</f>
+        <v/>
+      </c>
+      <c r="B14" s="37">
+        <f>Bordereau_prix!B6</f>
+        <v/>
+      </c>
+      <c r="C14" s="36">
+        <f>Bordereau_prix!C6</f>
+        <v/>
+      </c>
+      <c r="D14" s="36">
+        <f>Bordereau_prix!E6</f>
+        <v/>
+      </c>
+      <c r="E14" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A14)</f>
+        <v/>
+      </c>
+      <c r="F14" s="36">
+        <f>E14*D14</f>
+        <v/>
+      </c>
+      <c r="G14" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A14)</f>
+        <v/>
+      </c>
+      <c r="H14" s="36">
+        <f>G14*D14</f>
+        <v/>
+      </c>
+      <c r="I14" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A14)</f>
+        <v/>
+      </c>
+      <c r="J14" s="36">
+        <f>I14*D14</f>
+        <v/>
+      </c>
+      <c r="K14" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A14)</f>
+        <v/>
+      </c>
+      <c r="L14" s="36">
+        <f>K14*D14</f>
+        <v/>
+      </c>
+      <c r="M14" s="36">
+        <f>SUM(F14,H14,J14,L14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="36">
+        <f>Bordereau_prix!A7</f>
+        <v/>
+      </c>
+      <c r="B15" s="37">
+        <f>Bordereau_prix!B7</f>
+        <v/>
+      </c>
+      <c r="C15" s="36">
+        <f>Bordereau_prix!C7</f>
+        <v/>
+      </c>
+      <c r="D15" s="36">
+        <f>Bordereau_prix!E7</f>
+        <v/>
+      </c>
+      <c r="E15" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A15)</f>
+        <v/>
+      </c>
+      <c r="F15" s="36">
+        <f>E15*D15</f>
+        <v/>
+      </c>
+      <c r="G15" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A15)</f>
+        <v/>
+      </c>
+      <c r="H15" s="36">
+        <f>G15*D15</f>
+        <v/>
+      </c>
+      <c r="I15" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A15)</f>
+        <v/>
+      </c>
+      <c r="J15" s="36">
+        <f>I15*D15</f>
+        <v/>
+      </c>
+      <c r="K15" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A15)</f>
+        <v/>
+      </c>
+      <c r="L15" s="36">
+        <f>K15*D15</f>
+        <v/>
+      </c>
+      <c r="M15" s="36">
+        <f>SUM(F15,H15,J15,L15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="36">
+        <f>Bordereau_prix!A8</f>
+        <v/>
+      </c>
+      <c r="B16" s="37">
+        <f>Bordereau_prix!B8</f>
+        <v/>
+      </c>
+      <c r="C16" s="36">
+        <f>Bordereau_prix!C8</f>
+        <v/>
+      </c>
+      <c r="D16" s="36">
+        <f>Bordereau_prix!E8</f>
+        <v/>
+      </c>
+      <c r="E16" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A16)</f>
+        <v/>
+      </c>
+      <c r="F16" s="36">
+        <f>E16*D16</f>
+        <v/>
+      </c>
+      <c r="G16" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A16)</f>
+        <v/>
+      </c>
+      <c r="H16" s="36">
+        <f>G16*D16</f>
+        <v/>
+      </c>
+      <c r="I16" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A16)</f>
+        <v/>
+      </c>
+      <c r="J16" s="36">
+        <f>I16*D16</f>
+        <v/>
+      </c>
+      <c r="K16" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A16)</f>
+        <v/>
+      </c>
+      <c r="L16" s="36">
+        <f>K16*D16</f>
+        <v/>
+      </c>
+      <c r="M16" s="36">
+        <f>SUM(F16,H16,J16,L16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="36">
+        <f>Bordereau_prix!A9</f>
+        <v/>
+      </c>
+      <c r="B17" s="37">
+        <f>Bordereau_prix!B9</f>
+        <v/>
+      </c>
+      <c r="C17" s="36">
+        <f>Bordereau_prix!C9</f>
+        <v/>
+      </c>
+      <c r="D17" s="36">
+        <f>Bordereau_prix!E9</f>
+        <v/>
+      </c>
+      <c r="E17" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A17)</f>
+        <v/>
+      </c>
+      <c r="F17" s="36">
+        <f>E17*D17</f>
+        <v/>
+      </c>
+      <c r="G17" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A17)</f>
+        <v/>
+      </c>
+      <c r="H17" s="36">
+        <f>G17*D17</f>
+        <v/>
+      </c>
+      <c r="I17" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A17)</f>
+        <v/>
+      </c>
+      <c r="J17" s="36">
+        <f>I17*D17</f>
+        <v/>
+      </c>
+      <c r="K17" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A17)</f>
+        <v/>
+      </c>
+      <c r="L17" s="36">
+        <f>K17*D17</f>
+        <v/>
+      </c>
+      <c r="M17" s="36">
+        <f>SUM(F17,H17,J17,L17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="36">
+        <f>Bordereau_prix!A10</f>
+        <v/>
+      </c>
+      <c r="B18" s="37">
+        <f>Bordereau_prix!B10</f>
+        <v/>
+      </c>
+      <c r="C18" s="36">
+        <f>Bordereau_prix!C10</f>
+        <v/>
+      </c>
+      <c r="D18" s="36">
+        <f>Bordereau_prix!E10</f>
+        <v/>
+      </c>
+      <c r="E18" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A18)</f>
+        <v/>
+      </c>
+      <c r="F18" s="36">
+        <f>E18*D18</f>
+        <v/>
+      </c>
+      <c r="G18" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A18)</f>
+        <v/>
+      </c>
+      <c r="H18" s="36">
+        <f>G18*D18</f>
+        <v/>
+      </c>
+      <c r="I18" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A18)</f>
+        <v/>
+      </c>
+      <c r="J18" s="36">
+        <f>I18*D18</f>
+        <v/>
+      </c>
+      <c r="K18" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A18)</f>
+        <v/>
+      </c>
+      <c r="L18" s="36">
+        <f>K18*D18</f>
+        <v/>
+      </c>
+      <c r="M18" s="36">
+        <f>SUM(F18,H18,J18,L18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="36">
+        <f>Bordereau_prix!A11</f>
+        <v/>
+      </c>
+      <c r="B19" s="37">
+        <f>Bordereau_prix!B11</f>
+        <v/>
+      </c>
+      <c r="C19" s="36">
+        <f>Bordereau_prix!C11</f>
+        <v/>
+      </c>
+      <c r="D19" s="36">
+        <f>Bordereau_prix!E11</f>
+        <v/>
+      </c>
+      <c r="E19" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A19)</f>
+        <v/>
+      </c>
+      <c r="F19" s="36">
+        <f>E19*D19</f>
+        <v/>
+      </c>
+      <c r="G19" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A19)</f>
+        <v/>
+      </c>
+      <c r="H19" s="36">
+        <f>G19*D19</f>
+        <v/>
+      </c>
+      <c r="I19" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A19)</f>
+        <v/>
+      </c>
+      <c r="J19" s="36">
+        <f>I19*D19</f>
+        <v/>
+      </c>
+      <c r="K19" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A19)</f>
+        <v/>
+      </c>
+      <c r="L19" s="36">
+        <f>K19*D19</f>
+        <v/>
+      </c>
+      <c r="M19" s="36">
+        <f>SUM(F19,H19,J19,L19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="36">
+        <f>Bordereau_prix!A12</f>
+        <v/>
+      </c>
+      <c r="B20" s="37">
+        <f>Bordereau_prix!B12</f>
+        <v/>
+      </c>
+      <c r="C20" s="36">
+        <f>Bordereau_prix!C12</f>
+        <v/>
+      </c>
+      <c r="D20" s="36">
+        <f>Bordereau_prix!E12</f>
+        <v/>
+      </c>
+      <c r="E20" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A20)</f>
+        <v/>
+      </c>
+      <c r="F20" s="36">
+        <f>E20*D20</f>
+        <v/>
+      </c>
+      <c r="G20" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A20)</f>
+        <v/>
+      </c>
+      <c r="H20" s="36">
+        <f>G20*D20</f>
+        <v/>
+      </c>
+      <c r="I20" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A20)</f>
+        <v/>
+      </c>
+      <c r="J20" s="36">
+        <f>I20*D20</f>
+        <v/>
+      </c>
+      <c r="K20" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A20)</f>
+        <v/>
+      </c>
+      <c r="L20" s="36">
+        <f>K20*D20</f>
+        <v/>
+      </c>
+      <c r="M20" s="36">
+        <f>SUM(F20,H20,J20,L20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="36">
+        <f>Bordereau_prix!A13</f>
+        <v/>
+      </c>
+      <c r="B21" s="37">
+        <f>Bordereau_prix!B13</f>
+        <v/>
+      </c>
+      <c r="C21" s="36">
+        <f>Bordereau_prix!C13</f>
+        <v/>
+      </c>
+      <c r="D21" s="36">
+        <f>Bordereau_prix!E13</f>
+        <v/>
+      </c>
+      <c r="E21" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A21)</f>
+        <v/>
+      </c>
+      <c r="F21" s="36">
+        <f>E21*D21</f>
+        <v/>
+      </c>
+      <c r="G21" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A21)</f>
+        <v/>
+      </c>
+      <c r="H21" s="36">
+        <f>G21*D21</f>
+        <v/>
+      </c>
+      <c r="I21" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A21)</f>
+        <v/>
+      </c>
+      <c r="J21" s="36">
+        <f>I21*D21</f>
+        <v/>
+      </c>
+      <c r="K21" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A21)</f>
+        <v/>
+      </c>
+      <c r="L21" s="36">
+        <f>K21*D21</f>
+        <v/>
+      </c>
+      <c r="M21" s="36">
+        <f>SUM(F21,H21,J21,L21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="36">
+        <f>Bordereau_prix!A14</f>
+        <v/>
+      </c>
+      <c r="B22" s="37">
+        <f>Bordereau_prix!B14</f>
+        <v/>
+      </c>
+      <c r="C22" s="36">
+        <f>Bordereau_prix!C14</f>
+        <v/>
+      </c>
+      <c r="D22" s="36">
+        <f>Bordereau_prix!E14</f>
+        <v/>
+      </c>
+      <c r="E22" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A22)</f>
+        <v/>
+      </c>
+      <c r="F22" s="36">
+        <f>E22*D22</f>
+        <v/>
+      </c>
+      <c r="G22" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A22)</f>
+        <v/>
+      </c>
+      <c r="H22" s="36">
+        <f>G22*D22</f>
+        <v/>
+      </c>
+      <c r="I22" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A22)</f>
+        <v/>
+      </c>
+      <c r="J22" s="36">
+        <f>I22*D22</f>
+        <v/>
+      </c>
+      <c r="K22" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A22)</f>
+        <v/>
+      </c>
+      <c r="L22" s="36">
+        <f>K22*D22</f>
+        <v/>
+      </c>
+      <c r="M22" s="36">
+        <f>SUM(F22,H22,J22,L22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="36">
+        <f>Bordereau_prix!A15</f>
+        <v/>
+      </c>
+      <c r="B23" s="37">
+        <f>Bordereau_prix!B15</f>
+        <v/>
+      </c>
+      <c r="C23" s="36">
+        <f>Bordereau_prix!C15</f>
+        <v/>
+      </c>
+      <c r="D23" s="36">
+        <f>Bordereau_prix!E15</f>
+        <v/>
+      </c>
+      <c r="E23" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A23)</f>
+        <v/>
+      </c>
+      <c r="F23" s="36">
+        <f>E23*D23</f>
+        <v/>
+      </c>
+      <c r="G23" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A23)</f>
+        <v/>
+      </c>
+      <c r="H23" s="36">
+        <f>G23*D23</f>
+        <v/>
+      </c>
+      <c r="I23" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A23)</f>
+        <v/>
+      </c>
+      <c r="J23" s="36">
+        <f>I23*D23</f>
+        <v/>
+      </c>
+      <c r="K23" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A23)</f>
+        <v/>
+      </c>
+      <c r="L23" s="36">
+        <f>K23*D23</f>
+        <v/>
+      </c>
+      <c r="M23" s="36">
+        <f>SUM(F23,H23,J23,L23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="36">
+        <f>Bordereau_prix!A16</f>
+        <v/>
+      </c>
+      <c r="B24" s="37">
+        <f>Bordereau_prix!B16</f>
+        <v/>
+      </c>
+      <c r="C24" s="36">
+        <f>Bordereau_prix!C16</f>
+        <v/>
+      </c>
+      <c r="D24" s="36">
+        <f>Bordereau_prix!E16</f>
+        <v/>
+      </c>
+      <c r="E24" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A24)</f>
+        <v/>
+      </c>
+      <c r="F24" s="36">
+        <f>E24*D24</f>
+        <v/>
+      </c>
+      <c r="G24" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A24)</f>
+        <v/>
+      </c>
+      <c r="H24" s="36">
+        <f>G24*D24</f>
+        <v/>
+      </c>
+      <c r="I24" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A24)</f>
+        <v/>
+      </c>
+      <c r="J24" s="36">
+        <f>I24*D24</f>
+        <v/>
+      </c>
+      <c r="K24" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A24)</f>
+        <v/>
+      </c>
+      <c r="L24" s="36">
+        <f>K24*D24</f>
+        <v/>
+      </c>
+      <c r="M24" s="36">
+        <f>SUM(F24,H24,J24,L24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="36">
+        <f>Bordereau_prix!A17</f>
+        <v/>
+      </c>
+      <c r="B25" s="37">
+        <f>Bordereau_prix!B17</f>
+        <v/>
+      </c>
+      <c r="C25" s="36">
+        <f>Bordereau_prix!C17</f>
+        <v/>
+      </c>
+      <c r="D25" s="36">
+        <f>Bordereau_prix!E17</f>
+        <v/>
+      </c>
+      <c r="E25" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A25)</f>
+        <v/>
+      </c>
+      <c r="F25" s="36">
+        <f>E25*D25</f>
+        <v/>
+      </c>
+      <c r="G25" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A25)</f>
+        <v/>
+      </c>
+      <c r="H25" s="36">
+        <f>G25*D25</f>
+        <v/>
+      </c>
+      <c r="I25" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A25)</f>
+        <v/>
+      </c>
+      <c r="J25" s="36">
+        <f>I25*D25</f>
+        <v/>
+      </c>
+      <c r="K25" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A25)</f>
+        <v/>
+      </c>
+      <c r="L25" s="36">
+        <f>K25*D25</f>
+        <v/>
+      </c>
+      <c r="M25" s="36">
+        <f>SUM(F25,H25,J25,L25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="36">
+        <f>Bordereau_prix!A18</f>
+        <v/>
+      </c>
+      <c r="B26" s="37">
+        <f>Bordereau_prix!B18</f>
+        <v/>
+      </c>
+      <c r="C26" s="36">
+        <f>Bordereau_prix!C18</f>
+        <v/>
+      </c>
+      <c r="D26" s="36">
+        <f>Bordereau_prix!E18</f>
+        <v/>
+      </c>
+      <c r="E26" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A26)</f>
+        <v/>
+      </c>
+      <c r="F26" s="36">
+        <f>E26*D26</f>
+        <v/>
+      </c>
+      <c r="G26" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A26)</f>
+        <v/>
+      </c>
+      <c r="H26" s="36">
+        <f>G26*D26</f>
+        <v/>
+      </c>
+      <c r="I26" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A26)</f>
+        <v/>
+      </c>
+      <c r="J26" s="36">
+        <f>I26*D26</f>
+        <v/>
+      </c>
+      <c r="K26" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A26)</f>
+        <v/>
+      </c>
+      <c r="L26" s="36">
+        <f>K26*D26</f>
+        <v/>
+      </c>
+      <c r="M26" s="36">
+        <f>SUM(F26,H26,J26,L26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="36">
+        <f>Bordereau_prix!A19</f>
+        <v/>
+      </c>
+      <c r="B27" s="37">
+        <f>Bordereau_prix!B19</f>
+        <v/>
+      </c>
+      <c r="C27" s="36">
+        <f>Bordereau_prix!C19</f>
+        <v/>
+      </c>
+      <c r="D27" s="36">
+        <f>Bordereau_prix!E19</f>
+        <v/>
+      </c>
+      <c r="E27" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A27)</f>
+        <v/>
+      </c>
+      <c r="F27" s="36">
+        <f>E27*D27</f>
+        <v/>
+      </c>
+      <c r="G27" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A27)</f>
+        <v/>
+      </c>
+      <c r="H27" s="36">
+        <f>G27*D27</f>
+        <v/>
+      </c>
+      <c r="I27" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A27)</f>
+        <v/>
+      </c>
+      <c r="J27" s="36">
+        <f>I27*D27</f>
+        <v/>
+      </c>
+      <c r="K27" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A27)</f>
+        <v/>
+      </c>
+      <c r="L27" s="36">
+        <f>K27*D27</f>
+        <v/>
+      </c>
+      <c r="M27" s="36">
+        <f>SUM(F27,H27,J27,L27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="36">
+        <f>Bordereau_prix!A20</f>
+        <v/>
+      </c>
+      <c r="B28" s="37">
+        <f>Bordereau_prix!B20</f>
+        <v/>
+      </c>
+      <c r="C28" s="36">
+        <f>Bordereau_prix!C20</f>
+        <v/>
+      </c>
+      <c r="D28" s="36">
+        <f>Bordereau_prix!E20</f>
+        <v/>
+      </c>
+      <c r="E28" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A28)</f>
+        <v/>
+      </c>
+      <c r="F28" s="36">
+        <f>E28*D28</f>
+        <v/>
+      </c>
+      <c r="G28" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A28)</f>
+        <v/>
+      </c>
+      <c r="H28" s="36">
+        <f>G28*D28</f>
+        <v/>
+      </c>
+      <c r="I28" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A28)</f>
+        <v/>
+      </c>
+      <c r="J28" s="36">
+        <f>I28*D28</f>
+        <v/>
+      </c>
+      <c r="K28" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A28)</f>
+        <v/>
+      </c>
+      <c r="L28" s="36">
+        <f>K28*D28</f>
+        <v/>
+      </c>
+      <c r="M28" s="36">
+        <f>SUM(F28,H28,J28,L28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="36">
+        <f>Bordereau_prix!A21</f>
+        <v/>
+      </c>
+      <c r="B29" s="37">
+        <f>Bordereau_prix!B21</f>
+        <v/>
+      </c>
+      <c r="C29" s="36">
+        <f>Bordereau_prix!C21</f>
+        <v/>
+      </c>
+      <c r="D29" s="36">
+        <f>Bordereau_prix!E21</f>
+        <v/>
+      </c>
+      <c r="E29" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A29)</f>
+        <v/>
+      </c>
+      <c r="F29" s="36">
+        <f>E29*D29</f>
+        <v/>
+      </c>
+      <c r="G29" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A29)</f>
+        <v/>
+      </c>
+      <c r="H29" s="36">
+        <f>G29*D29</f>
+        <v/>
+      </c>
+      <c r="I29" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A29)</f>
+        <v/>
+      </c>
+      <c r="J29" s="36">
+        <f>I29*D29</f>
+        <v/>
+      </c>
+      <c r="K29" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A29)</f>
+        <v/>
+      </c>
+      <c r="L29" s="36">
+        <f>K29*D29</f>
+        <v/>
+      </c>
+      <c r="M29" s="36">
+        <f>SUM(F29,H29,J29,L29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="36">
+        <f>Bordereau_prix!A22</f>
+        <v/>
+      </c>
+      <c r="B30" s="37">
+        <f>Bordereau_prix!B22</f>
+        <v/>
+      </c>
+      <c r="C30" s="36">
+        <f>Bordereau_prix!C22</f>
+        <v/>
+      </c>
+      <c r="D30" s="36">
+        <f>Bordereau_prix!E22</f>
+        <v/>
+      </c>
+      <c r="E30" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A30)</f>
+        <v/>
+      </c>
+      <c r="F30" s="36">
+        <f>E30*D30</f>
+        <v/>
+      </c>
+      <c r="G30" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A30)</f>
+        <v/>
+      </c>
+      <c r="H30" s="36">
+        <f>G30*D30</f>
+        <v/>
+      </c>
+      <c r="I30" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A30)</f>
+        <v/>
+      </c>
+      <c r="J30" s="36">
+        <f>I30*D30</f>
+        <v/>
+      </c>
+      <c r="K30" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A30)</f>
+        <v/>
+      </c>
+      <c r="L30" s="36">
+        <f>K30*D30</f>
+        <v/>
+      </c>
+      <c r="M30" s="36">
+        <f>SUM(F30,H30,J30,L30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="36">
+        <f>Bordereau_prix!A23</f>
+        <v/>
+      </c>
+      <c r="B31" s="37">
+        <f>Bordereau_prix!B23</f>
+        <v/>
+      </c>
+      <c r="C31" s="36">
+        <f>Bordereau_prix!C23</f>
+        <v/>
+      </c>
+      <c r="D31" s="36">
+        <f>Bordereau_prix!E23</f>
+        <v/>
+      </c>
+      <c r="E31" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A31)</f>
+        <v/>
+      </c>
+      <c r="F31" s="36">
+        <f>E31*D31</f>
+        <v/>
+      </c>
+      <c r="G31" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A31)</f>
+        <v/>
+      </c>
+      <c r="H31" s="36">
+        <f>G31*D31</f>
+        <v/>
+      </c>
+      <c r="I31" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A31)</f>
+        <v/>
+      </c>
+      <c r="J31" s="36">
+        <f>I31*D31</f>
+        <v/>
+      </c>
+      <c r="K31" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A31)</f>
+        <v/>
+      </c>
+      <c r="L31" s="36">
+        <f>K31*D31</f>
+        <v/>
+      </c>
+      <c r="M31" s="36">
+        <f>SUM(F31,H31,J31,L31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="36">
+        <f>Bordereau_prix!A24</f>
+        <v/>
+      </c>
+      <c r="B32" s="37">
+        <f>Bordereau_prix!B24</f>
+        <v/>
+      </c>
+      <c r="C32" s="36">
+        <f>Bordereau_prix!C24</f>
+        <v/>
+      </c>
+      <c r="D32" s="36">
+        <f>Bordereau_prix!E24</f>
+        <v/>
+      </c>
+      <c r="E32" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A32)</f>
+        <v/>
+      </c>
+      <c r="F32" s="36">
+        <f>E32*D32</f>
+        <v/>
+      </c>
+      <c r="G32" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A32)</f>
+        <v/>
+      </c>
+      <c r="H32" s="36">
+        <f>G32*D32</f>
+        <v/>
+      </c>
+      <c r="I32" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A32)</f>
+        <v/>
+      </c>
+      <c r="J32" s="36">
+        <f>I32*D32</f>
+        <v/>
+      </c>
+      <c r="K32" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A32)</f>
+        <v/>
+      </c>
+      <c r="L32" s="36">
+        <f>K32*D32</f>
+        <v/>
+      </c>
+      <c r="M32" s="36">
+        <f>SUM(F32,H32,J32,L32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="36">
+        <f>Bordereau_prix!A25</f>
+        <v/>
+      </c>
+      <c r="B33" s="37">
+        <f>Bordereau_prix!B25</f>
+        <v/>
+      </c>
+      <c r="C33" s="36">
+        <f>Bordereau_prix!C25</f>
+        <v/>
+      </c>
+      <c r="D33" s="36">
+        <f>Bordereau_prix!E25</f>
+        <v/>
+      </c>
+      <c r="E33" s="36">
+        <f>SUMIFS('Secteur A'!$H:$H,'Secteur A'!$C:$C,$A33)</f>
+        <v/>
+      </c>
+      <c r="F33" s="36">
+        <f>E33*D33</f>
+        <v/>
+      </c>
+      <c r="G33" s="36">
+        <f>SUMIFS('Secteur P'!$H:$H,'Secteur P'!$C:$C,$A33)</f>
+        <v/>
+      </c>
+      <c r="H33" s="36">
+        <f>G33*D33</f>
+        <v/>
+      </c>
+      <c r="I33" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,$A33)</f>
+        <v/>
+      </c>
+      <c r="J33" s="36">
+        <f>I33*D33</f>
+        <v/>
+      </c>
+      <c r="K33" s="36">
+        <f>SUMIFS(Detail_facade_batim!$H:$H,Detail_facade_batim!$C:$C,$A33)</f>
+        <v/>
+      </c>
+      <c r="L33" s="36">
+        <f>K33*D33</f>
+        <v/>
+      </c>
+      <c r="M33" s="36">
+        <f>SUM(F33,H33,J33,L33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="32" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="F34" s="32">
+        <f>SUM(F13:F33)</f>
+        <v/>
+      </c>
+      <c r="H34" s="32">
+        <f>SUM(H13:H33)</f>
+        <v/>
+      </c>
+      <c r="J34" s="32">
+        <f>SUM(J13:J33)</f>
+        <v/>
+      </c>
+      <c r="L34" s="32">
+        <f>SUM(L13:L33)</f>
+        <v/>
+      </c>
+      <c r="M34" s="32">
+        <f>SUM(M13:M33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
+        <is>
+          <t>Note: cette feuille conserve la synthese globale et detaille la repartition des couts par secteur.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A36:M36"/>
+    <mergeCell ref="A1:M1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add sector drainage justifications and rename new catch basin items
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/Bordereau_prix_drainage_par_secteur.xlsx
+++ b/engineering/stormwater-pumping/Bordereau_prix_drainage_par_secteur.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Traceabilite" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Catalogue_items" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Estimation_par_secteur" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Justification_technique" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -166,7 +167,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -274,6 +275,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -942,12 +952,12 @@
     <row r="14" ht="15" customHeight="1" s="14">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>REG-001</t>
+          <t>PUI-010</t>
         </is>
       </c>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>Regard RP-01 (ajustement / reconstruction locale)</t>
+          <t>Nouveau puisard P-01</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
@@ -968,7 +978,7 @@
       </c>
       <c r="G14" s="21" t="inlineStr">
         <is>
-          <t>Noeud de repartition</t>
+          <t>Secteur Façade</t>
         </is>
       </c>
       <c r="H14" s="21" t="inlineStr">
@@ -980,12 +990,12 @@
     <row r="15" ht="15" customHeight="1" s="14">
       <c r="A15" s="20" t="inlineStr">
         <is>
-          <t>REG-002</t>
+          <t>PUI-020</t>
         </is>
       </c>
       <c r="B15" s="21" t="inlineStr">
         <is>
-          <t>Regard RP-02 avec clapet anti-retour</t>
+          <t>Nouveau puisard P-02</t>
         </is>
       </c>
       <c r="C15" s="20" t="inlineStr">
@@ -1006,7 +1016,7 @@
       </c>
       <c r="G15" s="21" t="inlineStr">
         <is>
-          <t>Aval poste / reseau existant</t>
+          <t>Secteur Façade</t>
         </is>
       </c>
       <c r="H15" s="21" t="inlineStr">
@@ -2444,12 +2454,12 @@
       </c>
       <c r="C7" s="20" t="inlineStr">
         <is>
-          <t>REG-001</t>
+          <t>PUI-010</t>
         </is>
       </c>
       <c r="D7" s="21" t="inlineStr">
         <is>
-          <t>Regard/interconnexion P-01</t>
+          <t>Nouveau puisard P-01</t>
         </is>
       </c>
       <c r="E7" s="20" t="inlineStr">
@@ -2487,12 +2497,12 @@
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>REG-002</t>
+          <t>PUI-020</t>
         </is>
       </c>
       <c r="D8" s="21" t="inlineStr">
         <is>
-          <t>Regard/interconnexion P-02</t>
+          <t>Nouveau puisard P-02</t>
         </is>
       </c>
       <c r="E8" s="20" t="inlineStr">
@@ -2772,7 +2782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="140" customWidth="1" style="13" min="1" max="1"/>
@@ -2873,6 +2883,20 @@
       <c r="A16" s="13" t="inlineStr">
         <is>
           <t>- La colonne PU contient des prix indicatifs Quebec (2025-2026) a valider par soumissions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>- Voir onglet Justification_technique pour le raisonnement hydraulique par secteur (A, P, Façade).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>- Les postes RP-01/RP-02 du bordereau ont ete renommes en nouveaux puisards P-01/P-02.</t>
         </is>
       </c>
     </row>
@@ -3121,12 +3145,12 @@
     <row r="11" ht="15" customHeight="1" s="14">
       <c r="A11" s="20" t="inlineStr">
         <is>
-          <t>REG-001</t>
+          <t>PUI-010</t>
         </is>
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>Regard RP-01 (ajustement / reconstruction locale)</t>
+          <t>Nouveau puisard P-01</t>
         </is>
       </c>
       <c r="C11" s="20" t="inlineStr">
@@ -3136,19 +3160,19 @@
       </c>
       <c r="D11" s="21" t="inlineStr">
         <is>
-          <t>Noeud de repartition</t>
+          <t>Secteur Façade</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="14">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t>REG-002</t>
+          <t>PUI-020</t>
         </is>
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>Regard RP-02 avec clapet anti-retour</t>
+          <t>Nouveau puisard P-02</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
@@ -3158,7 +3182,7 @@
       </c>
       <c r="D12" s="21" t="inlineStr">
         <is>
-          <t>Aval poste / reseau existant</t>
+          <t>Secteur Façade</t>
         </is>
       </c>
     </row>
@@ -4741,4 +4765,207 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" style="14" min="1" max="1"/>
+    <col width="44" customWidth="1" style="14" min="2" max="2"/>
+    <col width="42" customWidth="1" style="14" min="3" max="3"/>
+    <col width="42" customWidth="1" style="14" min="4" max="4"/>
+    <col width="46" customWidth="1" style="14" min="5" max="5"/>
+    <col width="38" customWidth="1" style="14" min="6" max="6"/>
+    <col width="36" customWidth="1" style="14" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>JUSTIFICATION TECHNIQUE - SOLUTIONS DE DRAINAGE PAR SECTEUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="35" t="inlineStr">
+        <is>
+          <t>Secteur</t>
+        </is>
+      </c>
+      <c r="B3" s="35" t="inlineStr">
+        <is>
+          <t>Problematique constatee</t>
+        </is>
+      </c>
+      <c r="C3" s="35" t="inlineStr">
+        <is>
+          <t>Principe de solution</t>
+        </is>
+      </c>
+      <c r="D3" s="35" t="inlineStr">
+        <is>
+          <t>Travaux proposes</t>
+        </is>
+      </c>
+      <c r="E3" s="35" t="inlineStr">
+        <is>
+          <t>Justification hydraulique</t>
+        </is>
+      </c>
+      <c r="F3" s="35" t="inlineStr">
+        <is>
+          <t>Resultat attendu</t>
+        </is>
+      </c>
+      <c r="G3" s="35" t="inlineStr">
+        <is>
+          <t>Points de validation terrain</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="38" t="inlineStr">
+        <is>
+          <t>Secteur A</t>
+        </is>
+      </c>
+      <c r="B4" s="39" t="inlineStr">
+        <is>
+          <t>Accumulation d'eau et risque d'inondation localisee au sud-ouest du batiment, en aval de la zone de reprofilage (zone identifiee 'A').</t>
+        </is>
+      </c>
+      <c r="C4" s="39" t="inlineStr">
+        <is>
+          <t>Corriger les pentes de surface pour eliminer le point bas actuel et evacuer le ruissellement vers le reseau pluvial plutot que vers la facade du batiment.</t>
+        </is>
+      </c>
+      <c r="D4" s="39" t="inlineStr">
+        <is>
+          <t>- Reprofilage de la surface pavee
+- Sciage et enlevement local du pavage si requis
+- Remblai/ajustement granulaire pour obtenir les nouvelles pentes
+- Refection finale des surfaces</t>
+        </is>
+      </c>
+      <c r="E4" s="39" t="inlineStr">
+        <is>
+          <t>La remise en pente diminue la hauteur d'eau stockee en surface et augmente la vitesse de drainage vers les exutoires. En supprimant la cuvette locale, on reduit la frequence de stagnation et de debordement vers le batiment.</t>
+        </is>
+      </c>
+      <c r="F4" s="39" t="inlineStr">
+        <is>
+          <t>Reduction significative des eaux de surface dirigees vers le batiment et disparition du point d'eau recurrent en condition de pluie courante.</t>
+        </is>
+      </c>
+      <c r="G4" s="39" t="inlineStr">
+        <is>
+          <t>- Validation altimetrique apres travaux
+- Verification des pentes minimales reelles
+- Arrosage/test pluie pour confirmer l'ecoulement</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="38" t="inlineStr">
+        <is>
+          <t>Secteur P</t>
+        </is>
+      </c>
+      <c r="B5" s="39" t="inlineStr">
+        <is>
+          <t>Probleme similaire de drainage de surface avec accumulation locale. Le ruissellement n'est pas capte efficacement dans l'etat actuel.</t>
+        </is>
+      </c>
+      <c r="C5" s="39" t="inlineStr">
+        <is>
+          <t>Creer un chemin hydraulique preferentiel vers un nouveau puisard par reprofilage des pentes et ouverture de bordure (saignee).</t>
+        </is>
+      </c>
+      <c r="D5" s="39" t="inlineStr">
+        <is>
+          <t>- Saignée dans bordure au nord de la zone problematique
+- Nouveau puisard (Secteur P)
+- Reprofilage des pentes vers le puisard
+- Ajustements connexes de surface</t>
+        </is>
+      </c>
+      <c r="E5" s="39" t="inlineStr">
+        <is>
+          <t>La saignee de bordure agit comme point d'entree gravitaire controle vers le systeme de captation. Le reprofilage assure une convergence des filets d'eau vers le puisard, ce qui reduit le volume en nappe sur la zone pavee.</t>
+        </is>
+      </c>
+      <c r="F5" s="39" t="inlineStr">
+        <is>
+          <t>Captage plus rapide des eaux de ruissellement et reduction des zones de stagnation en pied de pente.</t>
+        </is>
+      </c>
+      <c r="G5" s="39" t="inlineStr">
+        <is>
+          <t>- Cote d'entree de saignee
+- Capacite et niveau d'inversion du nouveau puisard
+- Verification des pentes transversales et longitudinales</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="38" t="inlineStr">
+        <is>
+          <t>Secteur Façade</t>
+        </is>
+      </c>
+      <c r="B6" s="39" t="inlineStr">
+        <is>
+          <t>Le ruissellement actuel tend a descendre vers l'avant du batiment (condition existante defavorable), avec risque de concentration d'eau en facade.</t>
+        </is>
+      </c>
+      <c r="C6" s="39" t="inlineStr">
+        <is>
+          <t>Inverser/reorienter l'ecoulement de surface pour eloigner l'eau de la facade et la capter par de nouveaux points de collecte.</t>
+        </is>
+      </c>
+      <c r="D6" s="39" t="inlineStr">
+        <is>
+          <t>- Installation de deux nouveaux puisards P-01 et P-02
+- Preparation/modelage de terrain dans la zone delimitee en rouge (facade-batim)
+- Raccordement du ruissellement vers les nouveaux puisards</t>
+        </is>
+      </c>
+      <c r="E6" s="39" t="inlineStr">
+        <is>
+          <t>Le double captage (P-01 et P-02) augmente la robustesse hydraulique locale et reduit la longueur de cheminement de l'eau vers un point d'entree. Le remodelage de terrain inverse la direction de pente dominante pour eviter la mise en charge de la facade.</t>
+        </is>
+      </c>
+      <c r="F6" s="39" t="inlineStr">
+        <is>
+          <t>Derivation du ruissellement a l'oppose de la facade et reduction du risque d'infiltration/accumulation au front du batiment.</t>
+        </is>
+      </c>
+      <c r="G6" s="39" t="inlineStr">
+        <is>
+          <t>- Releve final des cotes de surface en facade
+- Verification fonctionnelle des puisards P-01/P-02
+- Confirmation visuelle de la nouvelle direction d'ecoulement</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="40" t="inlineStr">
+        <is>
+          <t>Note: Cette justification accompagne le bordereau de prix et doit etre validee avec le releve final (topographie as-built) avant emission finale pour construction.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
add sector technical justifications and rename P-01/P-02 catch basin items
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/Bordereau_prix_drainage_par_secteur.xlsx
+++ b/engineering/stormwater-pumping/Bordereau_prix_drainage_par_secteur.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Traceabilite" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Catalogue_items" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Estimation_par_secteur" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Justification_technique" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -166,7 +167,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -274,6 +275,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -942,12 +952,12 @@
     <row r="14" ht="15" customHeight="1" s="14">
       <c r="A14" s="20" t="inlineStr">
         <is>
-          <t>REG-001</t>
+          <t>PUI-010</t>
         </is>
       </c>
       <c r="B14" s="21" t="inlineStr">
         <is>
-          <t>Regard RP-01 (ajustement / reconstruction locale)</t>
+          <t>Nouveau puisard P-01</t>
         </is>
       </c>
       <c r="C14" s="20" t="inlineStr">
@@ -968,7 +978,7 @@
       </c>
       <c r="G14" s="21" t="inlineStr">
         <is>
-          <t>Noeud de repartition</t>
+          <t>Secteur Façade</t>
         </is>
       </c>
       <c r="H14" s="21" t="inlineStr">
@@ -980,12 +990,12 @@
     <row r="15" ht="15" customHeight="1" s="14">
       <c r="A15" s="20" t="inlineStr">
         <is>
-          <t>REG-002</t>
+          <t>PUI-020</t>
         </is>
       </c>
       <c r="B15" s="21" t="inlineStr">
         <is>
-          <t>Regard RP-02 avec clapet anti-retour</t>
+          <t>Nouveau puisard P-02</t>
         </is>
       </c>
       <c r="C15" s="20" t="inlineStr">
@@ -1006,7 +1016,7 @@
       </c>
       <c r="G15" s="21" t="inlineStr">
         <is>
-          <t>Aval poste / reseau existant</t>
+          <t>Secteur Façade</t>
         </is>
       </c>
       <c r="H15" s="21" t="inlineStr">
@@ -2444,12 +2454,12 @@
       </c>
       <c r="C7" s="20" t="inlineStr">
         <is>
-          <t>REG-001</t>
+          <t>PUI-010</t>
         </is>
       </c>
       <c r="D7" s="21" t="inlineStr">
         <is>
-          <t>Regard/interconnexion P-01</t>
+          <t>Nouveau puisard P-01</t>
         </is>
       </c>
       <c r="E7" s="20" t="inlineStr">
@@ -2487,12 +2497,12 @@
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>REG-002</t>
+          <t>PUI-020</t>
         </is>
       </c>
       <c r="D8" s="21" t="inlineStr">
         <is>
-          <t>Regard/interconnexion P-02</t>
+          <t>Nouveau puisard P-02</t>
         </is>
       </c>
       <c r="E8" s="20" t="inlineStr">
@@ -2772,7 +2782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.54296875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="140" customWidth="1" style="13" min="1" max="1"/>
@@ -2873,6 +2883,20 @@
       <c r="A16" s="13" t="inlineStr">
         <is>
           <t>- La colonne PU contient des prix indicatifs Quebec (2025-2026) a valider par soumissions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>- Voir onglet Justification_technique pour le raisonnement hydraulique par secteur (A, P, Façade).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>- Les postes RP-01/RP-02 du bordereau ont ete renommes en nouveaux puisards P-01/P-02.</t>
         </is>
       </c>
     </row>
@@ -3121,12 +3145,12 @@
     <row r="11" ht="15" customHeight="1" s="14">
       <c r="A11" s="20" t="inlineStr">
         <is>
-          <t>REG-001</t>
+          <t>PUI-010</t>
         </is>
       </c>
       <c r="B11" s="21" t="inlineStr">
         <is>
-          <t>Regard RP-01 (ajustement / reconstruction locale)</t>
+          <t>Nouveau puisard P-01</t>
         </is>
       </c>
       <c r="C11" s="20" t="inlineStr">
@@ -3136,19 +3160,19 @@
       </c>
       <c r="D11" s="21" t="inlineStr">
         <is>
-          <t>Noeud de repartition</t>
+          <t>Secteur Façade</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="14">
       <c r="A12" s="20" t="inlineStr">
         <is>
-          <t>REG-002</t>
+          <t>PUI-020</t>
         </is>
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>Regard RP-02 avec clapet anti-retour</t>
+          <t>Nouveau puisard P-02</t>
         </is>
       </c>
       <c r="C12" s="20" t="inlineStr">
@@ -3158,7 +3182,7 @@
       </c>
       <c r="D12" s="21" t="inlineStr">
         <is>
-          <t>Aval poste / reseau existant</t>
+          <t>Secteur Façade</t>
         </is>
       </c>
     </row>
@@ -4741,4 +4765,207 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" style="14" min="1" max="1"/>
+    <col width="44" customWidth="1" style="14" min="2" max="2"/>
+    <col width="42" customWidth="1" style="14" min="3" max="3"/>
+    <col width="42" customWidth="1" style="14" min="4" max="4"/>
+    <col width="46" customWidth="1" style="14" min="5" max="5"/>
+    <col width="38" customWidth="1" style="14" min="6" max="6"/>
+    <col width="36" customWidth="1" style="14" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="27" t="inlineStr">
+        <is>
+          <t>JUSTIFICATION TECHNIQUE - SOLUTIONS DE DRAINAGE PAR SECTEUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="35" t="inlineStr">
+        <is>
+          <t>Secteur</t>
+        </is>
+      </c>
+      <c r="B3" s="35" t="inlineStr">
+        <is>
+          <t>Problematique constatee</t>
+        </is>
+      </c>
+      <c r="C3" s="35" t="inlineStr">
+        <is>
+          <t>Principe de solution</t>
+        </is>
+      </c>
+      <c r="D3" s="35" t="inlineStr">
+        <is>
+          <t>Travaux proposes</t>
+        </is>
+      </c>
+      <c r="E3" s="35" t="inlineStr">
+        <is>
+          <t>Justification hydraulique</t>
+        </is>
+      </c>
+      <c r="F3" s="35" t="inlineStr">
+        <is>
+          <t>Resultat attendu</t>
+        </is>
+      </c>
+      <c r="G3" s="35" t="inlineStr">
+        <is>
+          <t>Points de validation terrain</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="38" t="inlineStr">
+        <is>
+          <t>Secteur A</t>
+        </is>
+      </c>
+      <c r="B4" s="39" t="inlineStr">
+        <is>
+          <t>Accumulation d'eau et risque d'inondation localisee au sud-ouest du batiment, en aval de la zone de reprofilage (zone identifiee 'A').</t>
+        </is>
+      </c>
+      <c r="C4" s="39" t="inlineStr">
+        <is>
+          <t>Corriger les pentes de surface pour eliminer le point bas actuel et evacuer le ruissellement vers le reseau pluvial plutot que vers la facade du batiment.</t>
+        </is>
+      </c>
+      <c r="D4" s="39" t="inlineStr">
+        <is>
+          <t>- Reprofilage de la surface pavee
+- Sciage et enlevement local du pavage si requis
+- Remblai/ajustement granulaire pour obtenir les nouvelles pentes
+- Refection finale des surfaces</t>
+        </is>
+      </c>
+      <c r="E4" s="39" t="inlineStr">
+        <is>
+          <t>La remise en pente diminue la hauteur d'eau stockee en surface et augmente la vitesse de drainage vers les exutoires. En supprimant la cuvette locale, on reduit la frequence de stagnation et de debordement vers le batiment.</t>
+        </is>
+      </c>
+      <c r="F4" s="39" t="inlineStr">
+        <is>
+          <t>Reduction significative des eaux de surface dirigees vers le batiment et disparition du point d'eau recurrent en condition de pluie courante.</t>
+        </is>
+      </c>
+      <c r="G4" s="39" t="inlineStr">
+        <is>
+          <t>- Validation altimetrique apres travaux
+- Verification des pentes minimales reelles
+- Arrosage/test pluie pour confirmer l'ecoulement</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="38" t="inlineStr">
+        <is>
+          <t>Secteur P</t>
+        </is>
+      </c>
+      <c r="B5" s="39" t="inlineStr">
+        <is>
+          <t>Probleme similaire de drainage de surface avec accumulation locale. Le ruissellement n'est pas capte efficacement dans l'etat actuel.</t>
+        </is>
+      </c>
+      <c r="C5" s="39" t="inlineStr">
+        <is>
+          <t>Creer un chemin hydraulique preferentiel vers un nouveau puisard par reprofilage des pentes et ouverture de bordure (saignee).</t>
+        </is>
+      </c>
+      <c r="D5" s="39" t="inlineStr">
+        <is>
+          <t>- Saignée dans bordure au nord de la zone problematique
+- Nouveau puisard (Secteur P)
+- Reprofilage des pentes vers le puisard
+- Ajustements connexes de surface</t>
+        </is>
+      </c>
+      <c r="E5" s="39" t="inlineStr">
+        <is>
+          <t>La saignee de bordure agit comme point d'entree gravitaire controle vers le systeme de captation. Le reprofilage assure une convergence des filets d'eau vers le puisard, ce qui reduit le volume en nappe sur la zone pavee.</t>
+        </is>
+      </c>
+      <c r="F5" s="39" t="inlineStr">
+        <is>
+          <t>Captage plus rapide des eaux de ruissellement et reduction des zones de stagnation en pied de pente.</t>
+        </is>
+      </c>
+      <c r="G5" s="39" t="inlineStr">
+        <is>
+          <t>- Cote d'entree de saignee
+- Capacite et niveau d'inversion du nouveau puisard
+- Verification des pentes transversales et longitudinales</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="38" t="inlineStr">
+        <is>
+          <t>Secteur Façade</t>
+        </is>
+      </c>
+      <c r="B6" s="39" t="inlineStr">
+        <is>
+          <t>Le ruissellement actuel tend a descendre vers l'avant du batiment (condition existante defavorable), avec risque de concentration d'eau en facade.</t>
+        </is>
+      </c>
+      <c r="C6" s="39" t="inlineStr">
+        <is>
+          <t>Inverser/reorienter l'ecoulement de surface pour eloigner l'eau de la facade et la capter par de nouveaux points de collecte.</t>
+        </is>
+      </c>
+      <c r="D6" s="39" t="inlineStr">
+        <is>
+          <t>- Installation de deux nouveaux puisards P-01 et P-02
+- Preparation/modelage de terrain dans la zone delimitee en rouge (facade-batim)
+- Raccordement du ruissellement vers les nouveaux puisards</t>
+        </is>
+      </c>
+      <c r="E6" s="39" t="inlineStr">
+        <is>
+          <t>Le double captage (P-01 et P-02) augmente la robustesse hydraulique locale et reduit la longueur de cheminement de l'eau vers un point d'entree. Le remodelage de terrain inverse la direction de pente dominante pour eviter la mise en charge de la facade.</t>
+        </is>
+      </c>
+      <c r="F6" s="39" t="inlineStr">
+        <is>
+          <t>Derivation du ruissellement a l'oppose de la facade et reduction du risque d'infiltration/accumulation au front du batiment.</t>
+        </is>
+      </c>
+      <c r="G6" s="39" t="inlineStr">
+        <is>
+          <t>- Releve final des cotes de surface en facade
+- Verification fonctionnelle des puisards P-01/P-02
+- Confirmation visuelle de la nouvelle direction d'ecoulement</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="40" t="inlineStr">
+        <is>
+          <t>Note: Cette justification accompagne le bordereau de prix et doit etre validee avec le releve final (topographie as-built) avant emission finale pour construction.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A8:G8"/>
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add explicit facade code breakdown including EXC-002
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/Bordereau_prix_drainage_par_secteur.xlsx
+++ b/engineering/stormwater-pumping/Bordereau_prix_drainage_par_secteur.xlsx
@@ -167,7 +167,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -284,6 +284,12 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2887,14 +2893,14 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>- Voir onglet Justification_technique pour le raisonnement hydraulique par secteur (A, P, Façade).</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>- Les postes RP-01/RP-02 du bordereau ont ete renommes en nouveaux puisards P-01/P-02.</t>
         </is>
@@ -3425,7 +3431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="14" min="1" max="1"/>
@@ -3456,6 +3462,14 @@
           <t>Synthese des couts par secteur (CAD)</t>
         </is>
       </c>
+      <c r="D3" s="31" t="inlineStr">
+        <is>
+          <t>Verification Façade (reseau) par code</t>
+        </is>
+      </c>
+      <c r="E3" s="41" t="n"/>
+      <c r="F3" s="41" t="n"/>
+      <c r="G3" s="41" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="29" t="inlineStr">
@@ -3467,6 +3481,26 @@
         <f>SUM(F13:F33)</f>
         <v/>
       </c>
+      <c r="D4" s="35" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="E4" s="35" t="inlineStr">
+        <is>
+          <t>Qte_Façade</t>
+        </is>
+      </c>
+      <c r="F4" s="35" t="inlineStr">
+        <is>
+          <t>PU</t>
+        </is>
+      </c>
+      <c r="G4" s="35" t="inlineStr">
+        <is>
+          <t>Cout</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="29" t="inlineStr">
@@ -3478,6 +3512,23 @@
         <f>SUM(H13:H33)</f>
         <v/>
       </c>
+      <c r="D5" s="36" t="inlineStr">
+        <is>
+          <t>EXC-002</t>
+        </is>
+      </c>
+      <c r="E5" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,D5)</f>
+        <v/>
+      </c>
+      <c r="F5" s="36">
+        <f>IFERROR(INDEX(Bordereau_prix!$E$5:$E$25,MATCH(D5,Bordereau_prix!$A$5:$A$25,0)),0)</f>
+        <v/>
+      </c>
+      <c r="G5" s="36">
+        <f>E5*F5</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="29" t="inlineStr">
@@ -3489,6 +3540,23 @@
         <f>SUM(J13:J33)</f>
         <v/>
       </c>
+      <c r="D6" s="36" t="inlineStr">
+        <is>
+          <t>RAC-001</t>
+        </is>
+      </c>
+      <c r="E6" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,D6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="36">
+        <f>IFERROR(INDEX(Bordereau_prix!$E$5:$E$25,MATCH(D6,Bordereau_prix!$A$5:$A$25,0)),0)</f>
+        <v/>
+      </c>
+      <c r="G6" s="36">
+        <f>E6*F6</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="29" t="inlineStr">
@@ -3500,6 +3568,23 @@
         <f>SUM(L13:L33)</f>
         <v/>
       </c>
+      <c r="D7" s="36" t="inlineStr">
+        <is>
+          <t>CAN-300</t>
+        </is>
+      </c>
+      <c r="E7" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,D7)</f>
+        <v/>
+      </c>
+      <c r="F7" s="36">
+        <f>IFERROR(INDEX(Bordereau_prix!$E$5:$E$25,MATCH(D7,Bordereau_prix!$A$5:$A$25,0)),0)</f>
+        <v/>
+      </c>
+      <c r="G7" s="36">
+        <f>E7*F7</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="31" t="inlineStr">
@@ -3511,6 +3596,23 @@
         <f>SUM(B4:B7)</f>
         <v/>
       </c>
+      <c r="D8" s="36" t="inlineStr">
+        <is>
+          <t>PUI-010</t>
+        </is>
+      </c>
+      <c r="E8" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,D8)</f>
+        <v/>
+      </c>
+      <c r="F8" s="36">
+        <f>IFERROR(INDEX(Bordereau_prix!$E$5:$E$25,MATCH(D8,Bordereau_prix!$A$5:$A$25,0)),0)</f>
+        <v/>
+      </c>
+      <c r="G8" s="36">
+        <f>E8*F8</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="33" t="inlineStr">
@@ -3520,6 +3622,55 @@
       </c>
       <c r="B9" s="34">
         <f>B8-Bordereau_prix!F27</f>
+        <v/>
+      </c>
+      <c r="D9" s="36" t="inlineStr">
+        <is>
+          <t>PUI-020</t>
+        </is>
+      </c>
+      <c r="E9" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,D9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="36">
+        <f>IFERROR(INDEX(Bordereau_prix!$E$5:$E$25,MATCH(D9,Bordereau_prix!$A$5:$A$25,0)),0)</f>
+        <v/>
+      </c>
+      <c r="G9" s="36">
+        <f>E9*F9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="D10" s="36" t="inlineStr">
+        <is>
+          <t>EXC-001</t>
+        </is>
+      </c>
+      <c r="E10" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,D10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="36">
+        <f>IFERROR(INDEX(Bordereau_prix!$E$5:$E$25,MATCH(D10,Bordereau_prix!$A$5:$A$25,0)),0)</f>
+        <v/>
+      </c>
+      <c r="G10" s="36">
+        <f>E10*F10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="D11" s="42" t="inlineStr">
+        <is>
+          <t>Sous-total Façade (reseau)</t>
+        </is>
+      </c>
+      <c r="E11" s="43" t="n"/>
+      <c r="F11" s="43" t="n"/>
+      <c r="G11" s="42">
+        <f>SUM(G5:G10)</f>
         <v/>
       </c>
     </row>
@@ -4758,10 +4909,19 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="44" t="inlineStr">
+        <is>
+          <t>Controle: EXC-002 (Hydro-excavation) est comptabilise dans le Cout_Façade via l'onglet Façade.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="A36:M36"/>
+    <mergeCell ref="D3:G3"/>
     <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A37:M37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
make EXC-002 explicit in facade sector estimation
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/Bordereau_prix_drainage_par_secteur.xlsx
+++ b/engineering/stormwater-pumping/Bordereau_prix_drainage_par_secteur.xlsx
@@ -167,7 +167,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -284,6 +284,12 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2887,14 +2893,14 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>- Voir onglet Justification_technique pour le raisonnement hydraulique par secteur (A, P, Façade).</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>- Les postes RP-01/RP-02 du bordereau ont ete renommes en nouveaux puisards P-01/P-02.</t>
         </is>
@@ -3425,7 +3431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="14" min="1" max="1"/>
@@ -3456,6 +3462,14 @@
           <t>Synthese des couts par secteur (CAD)</t>
         </is>
       </c>
+      <c r="D3" s="31" t="inlineStr">
+        <is>
+          <t>Verification Façade (reseau) par code</t>
+        </is>
+      </c>
+      <c r="E3" s="41" t="n"/>
+      <c r="F3" s="41" t="n"/>
+      <c r="G3" s="41" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="29" t="inlineStr">
@@ -3467,6 +3481,26 @@
         <f>SUM(F13:F33)</f>
         <v/>
       </c>
+      <c r="D4" s="35" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="E4" s="35" t="inlineStr">
+        <is>
+          <t>Qte_Façade</t>
+        </is>
+      </c>
+      <c r="F4" s="35" t="inlineStr">
+        <is>
+          <t>PU</t>
+        </is>
+      </c>
+      <c r="G4" s="35" t="inlineStr">
+        <is>
+          <t>Cout</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="29" t="inlineStr">
@@ -3478,6 +3512,23 @@
         <f>SUM(H13:H33)</f>
         <v/>
       </c>
+      <c r="D5" s="36" t="inlineStr">
+        <is>
+          <t>EXC-002</t>
+        </is>
+      </c>
+      <c r="E5" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,D5)</f>
+        <v/>
+      </c>
+      <c r="F5" s="36">
+        <f>IFERROR(INDEX(Bordereau_prix!$E$5:$E$25,MATCH(D5,Bordereau_prix!$A$5:$A$25,0)),0)</f>
+        <v/>
+      </c>
+      <c r="G5" s="36">
+        <f>E5*F5</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="29" t="inlineStr">
@@ -3489,6 +3540,23 @@
         <f>SUM(J13:J33)</f>
         <v/>
       </c>
+      <c r="D6" s="36" t="inlineStr">
+        <is>
+          <t>RAC-001</t>
+        </is>
+      </c>
+      <c r="E6" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,D6)</f>
+        <v/>
+      </c>
+      <c r="F6" s="36">
+        <f>IFERROR(INDEX(Bordereau_prix!$E$5:$E$25,MATCH(D6,Bordereau_prix!$A$5:$A$25,0)),0)</f>
+        <v/>
+      </c>
+      <c r="G6" s="36">
+        <f>E6*F6</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="29" t="inlineStr">
@@ -3500,6 +3568,23 @@
         <f>SUM(L13:L33)</f>
         <v/>
       </c>
+      <c r="D7" s="36" t="inlineStr">
+        <is>
+          <t>CAN-300</t>
+        </is>
+      </c>
+      <c r="E7" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,D7)</f>
+        <v/>
+      </c>
+      <c r="F7" s="36">
+        <f>IFERROR(INDEX(Bordereau_prix!$E$5:$E$25,MATCH(D7,Bordereau_prix!$A$5:$A$25,0)),0)</f>
+        <v/>
+      </c>
+      <c r="G7" s="36">
+        <f>E7*F7</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="31" t="inlineStr">
@@ -3511,6 +3596,23 @@
         <f>SUM(B4:B7)</f>
         <v/>
       </c>
+      <c r="D8" s="36" t="inlineStr">
+        <is>
+          <t>PUI-010</t>
+        </is>
+      </c>
+      <c r="E8" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,D8)</f>
+        <v/>
+      </c>
+      <c r="F8" s="36">
+        <f>IFERROR(INDEX(Bordereau_prix!$E$5:$E$25,MATCH(D8,Bordereau_prix!$A$5:$A$25,0)),0)</f>
+        <v/>
+      </c>
+      <c r="G8" s="36">
+        <f>E8*F8</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="33" t="inlineStr">
@@ -3520,6 +3622,55 @@
       </c>
       <c r="B9" s="34">
         <f>B8-Bordereau_prix!F27</f>
+        <v/>
+      </c>
+      <c r="D9" s="36" t="inlineStr">
+        <is>
+          <t>PUI-020</t>
+        </is>
+      </c>
+      <c r="E9" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,D9)</f>
+        <v/>
+      </c>
+      <c r="F9" s="36">
+        <f>IFERROR(INDEX(Bordereau_prix!$E$5:$E$25,MATCH(D9,Bordereau_prix!$A$5:$A$25,0)),0)</f>
+        <v/>
+      </c>
+      <c r="G9" s="36">
+        <f>E9*F9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="D10" s="36" t="inlineStr">
+        <is>
+          <t>EXC-001</t>
+        </is>
+      </c>
+      <c r="E10" s="36">
+        <f>SUMIFS(Façade!$H:$H,Façade!$C:$C,D10)</f>
+        <v/>
+      </c>
+      <c r="F10" s="36">
+        <f>IFERROR(INDEX(Bordereau_prix!$E$5:$E$25,MATCH(D10,Bordereau_prix!$A$5:$A$25,0)),0)</f>
+        <v/>
+      </c>
+      <c r="G10" s="36">
+        <f>E10*F10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="D11" s="42" t="inlineStr">
+        <is>
+          <t>Sous-total Façade (reseau)</t>
+        </is>
+      </c>
+      <c r="E11" s="43" t="n"/>
+      <c r="F11" s="43" t="n"/>
+      <c r="G11" s="42">
+        <f>SUM(G5:G10)</f>
         <v/>
       </c>
     </row>
@@ -4758,10 +4909,19 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" s="44" t="inlineStr">
+        <is>
+          <t>Controle: EXC-002 (Hydro-excavation) est comptabilise dans le Cout_Façade via l'onglet Façade.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="A36:M36"/>
+    <mergeCell ref="D3:G3"/>
     <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A37:M37"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Refine Secteur P with separate sciage/demo/pavage/gazon items
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/stormwater-pumping/Bordereau_prix_drainage_par_secteur.xlsx
+++ b/engineering/stormwater-pumping/Bordereau_prix_drainage_par_secteur.xlsx
@@ -119,7 +119,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -156,6 +156,50 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -167,7 +211,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -291,6 +335,8 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1969,17 +2015,17 @@
       </c>
       <c r="B4" s="21" t="inlineStr">
         <is>
-          <t>Secteur P haut</t>
+          <t>Secteur P haut (gazon)</t>
         </is>
       </c>
       <c r="C4" s="20" t="inlineStr">
         <is>
-          <t>PAV-001</t>
+          <t>REF-001</t>
         </is>
       </c>
       <c r="D4" s="21" t="inlineStr">
         <is>
-          <t>Reprofilage / reprise de pavage</t>
+          <t>Refection des surfaces (gazon, etc.)</t>
         </is>
       </c>
       <c r="E4" s="20" t="inlineStr">
@@ -2012,7 +2058,7 @@
       </c>
       <c r="B5" s="21" t="inlineStr">
         <is>
-          <t>Secteur P bas</t>
+          <t>Secteur P bas (pavage)</t>
         </is>
       </c>
       <c r="C5" s="20" t="inlineStr">
@@ -2055,26 +2101,26 @@
       </c>
       <c r="B6" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Secteur P </t>
+          <t>Secteur P bas (pavage)</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
         <is>
-          <t>PUI-001</t>
+          <t>DEM-001</t>
         </is>
       </c>
       <c r="D6" s="21" t="inlineStr">
         <is>
-          <t>Nouveau puisard</t>
+          <t>Enlevement de pavage</t>
         </is>
       </c>
       <c r="E6" s="20" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="F6" s="20" t="n">
-        <v>1</v>
+        <v>80</v>
       </c>
       <c r="G6" s="20" t="n">
         <v>1</v>
@@ -2098,17 +2144,17 @@
       </c>
       <c r="B7" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Secteur P </t>
+          <t>Secteur P bas (pavage)</t>
         </is>
       </c>
       <c r="C7" s="20" t="inlineStr">
         <is>
-          <t>CAN-375</t>
+          <t>SCI-001</t>
         </is>
       </c>
       <c r="D7" s="21" t="inlineStr">
         <is>
-          <t>Raccord propose Ø375</t>
+          <t>Sciage de pavage</t>
         </is>
       </c>
       <c r="E7" s="20" t="inlineStr">
@@ -2116,9 +2162,7 @@
           <t>m</t>
         </is>
       </c>
-      <c r="F7" s="20" t="n">
-        <v>0</v>
-      </c>
+      <c r="F7" s="20" t="n"/>
       <c r="G7" s="20" t="n">
         <v>1</v>
       </c>
@@ -2141,26 +2185,26 @@
       </c>
       <c r="B8" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Secteur P </t>
+          <t>Secteur P</t>
         </is>
       </c>
       <c r="C8" s="20" t="inlineStr">
         <is>
-          <t>BOR-001</t>
+          <t>PUI-001</t>
         </is>
       </c>
       <c r="D8" s="21" t="inlineStr">
         <is>
-          <t>Saignee dans bordure</t>
+          <t>Nouveau puisard</t>
         </is>
       </c>
       <c r="E8" s="20" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>u</t>
         </is>
       </c>
       <c r="F8" s="20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" s="20" t="n">
         <v>1</v>
@@ -2184,26 +2228,26 @@
       </c>
       <c r="B9" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Secteur P </t>
+          <t>Secteur P</t>
         </is>
       </c>
       <c r="C9" s="20" t="inlineStr">
         <is>
-          <t>DEM-001</t>
+          <t>CAN-375</t>
         </is>
       </c>
       <c r="D9" s="21" t="inlineStr">
         <is>
-          <t>Decoupage/demolition de pavage</t>
+          <t>Raccord propose Ø375</t>
         </is>
       </c>
       <c r="E9" s="20" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>m</t>
         </is>
       </c>
       <c r="F9" s="20" t="n">
-        <v>164</v>
+        <v>0</v>
       </c>
       <c r="G9" s="20" t="n">
         <v>1</v>
@@ -2219,6 +2263,43 @@
       </c>
       <c r="J9" s="21" t="n"/>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>saignée.png</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Secteur P</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>BOR-001</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Saignee dans bordure</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10">
+        <f>IF(F10="","",F10*G10)</f>
+        <v/>
+      </c>
+    </row>
     <row r="11" ht="15" customHeight="1" s="14">
       <c r="A11" s="26" t="inlineStr">
         <is>
@@ -2226,7 +2307,7 @@
         </is>
       </c>
       <c r="H11" s="26">
-        <f>SUM(H4:H9)</f>
+        <f>SUM(H4:H10)</f>
         <v/>
       </c>
     </row>
@@ -3467,9 +3548,9 @@
           <t>Verification Façade (reseau) par code</t>
         </is>
       </c>
-      <c r="E3" s="41" t="n"/>
-      <c r="F3" s="41" t="n"/>
-      <c r="G3" s="41" t="n"/>
+      <c r="E3" s="45" t="n"/>
+      <c r="F3" s="45" t="n"/>
+      <c r="G3" s="46" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="29" t="inlineStr">

</xml_diff>